<commit_message>
Update subjective severity of potentially traumatic experience in TSO classes.xlsx
</commit_message>
<xml_diff>
--- a/TSO classes.xlsx
+++ b/TSO classes.xlsx
@@ -452,87 +452,87 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Parent</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Definition</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Parent</t>
-        </is>
-      </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Synonyms</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>BFO Entity</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Curation status</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Reviewer query</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Entity URL</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Sub-ontology</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Curation note</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Informal definition</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Fuzzy class</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Logical definition</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>BFO Entity</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Sub-ontology</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Synonyms</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Entity URL</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Curation status</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Curation note</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Comment</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Fuzzy class</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Curator</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Reviewer</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Why fuzzy</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Curator</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Reviewer</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Reviewer query</t>
         </is>
       </c>
     </row>
@@ -549,22 +549,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>potentially traumatic experience attribute</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>A &lt;potentially traumatic experience attribute&gt; that is whether event(s) were physically experienced, witnessed, or communicated to the person.</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience attribute</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>dimension</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
         <is>
           <t xml:space="preserve">The directness of a person's exposure to a potentially traumatic experience ranges from direct physical impact to one's body, to personally witnessing (seeing, hearing) event(s), to learning about event(s) that happened to other persons (loved ones or others). </t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>dimension</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -586,34 +586,34 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
+          <t>potentially traumatic experience</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>A &lt;potentially traumatic experience&gt; that involves actual (or potential) injury, without human intention to cause harm, and impacts one or a few people.</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Something that happens which causes potential or actual unintended harm.  Note that DISASTERS are similar but usually impact more people and often (not always) natural forces.</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>includes sub-classes for road traffic accident, fall, animal attack, residential fire, sports-related, weapon-related (unintentional), choking, drowning</t>
+        </is>
+      </c>
       <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="I3" s="2" t="n"/>
       <c r="J3" s="2" t="n"/>
       <c r="K3" s="2" t="n"/>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="L3" s="2" t="n"/>
       <c r="M3" s="2" t="n"/>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>includes sub-classes for road traffic accident, fall, animal attack, residential fire, sports-related, weapon-related (unintentional), choking, drowning</t>
+          <t>Something that happens which causes potential or actual unintended harm.  Note that DISASTERS are similar but usually impact more people and often (not always) natural forces.</t>
         </is>
       </c>
       <c r="O3" s="2" t="n"/>
@@ -639,32 +639,32 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
+          <t>potentially traumatic experience</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
           <t>A &lt;potentially traumatic experience&gt; that involves armed conflict between states or other military groups.</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience</t>
-        </is>
-      </c>
       <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>includes sub-classes for civilian exposure to warfare or armed conflict, combat exposure as a member of armed forces, deployment as a member of armed forces</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="n"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="I4" s="2" t="n"/>
       <c r="J4" s="2" t="n"/>
       <c r="K4" s="2" t="n"/>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="L4" s="2" t="n"/>
       <c r="M4" s="2" t="n"/>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>includes sub-classes for civilian exposure to warfare or armed conflict, combat exposure as a member of armed forces, deployment as a member of armed forces</t>
-        </is>
-      </c>
+      <c r="N4" s="2" t="n"/>
       <c r="O4" s="2" t="n"/>
       <c r="P4" s="2" t="n"/>
       <c r="Q4" s="2" t="inlineStr">
@@ -688,32 +688,32 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
+          <t>potentially traumatic experience</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
           <t>A &lt;potentially traumatic experience&gt; that is the death of a loved one.</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience</t>
-        </is>
-      </c>
       <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>need to consult with colleages about sub-classes - probably traumatic bereavement and others</t>
+        </is>
+      </c>
       <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
       <c r="K5" s="3" t="n"/>
-      <c r="L5" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
+      <c r="L5" s="3" t="n"/>
       <c r="M5" s="3" t="n"/>
-      <c r="N5" s="3" t="inlineStr">
-        <is>
-          <t>need to consult with colleages about sub-classes - probably traumatic bereavement and others</t>
-        </is>
-      </c>
+      <c r="N5" s="3" t="n"/>
       <c r="O5" s="3" t="n"/>
       <c r="P5" s="3" t="n"/>
       <c r="Q5" s="3" t="inlineStr">
@@ -725,7 +725,11 @@
       <c r="S5" s="3" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n"/>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>_:vis-5</t>
+        </is>
+      </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
           <t>experience of disaster</t>
@@ -733,32 +737,32 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
+          <t>potentially traumatic experience</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
           <t>A &lt;potentially traumatic experience&gt; that involves a sudden-onset occurrence created by natural or technological forces impacting a group of people defined by place or region</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience</t>
-        </is>
-      </c>
       <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>includes sub-classes for natural disaster, technological disaster, transportation disaster (and each of those has multiple sub-classes)</t>
+        </is>
+      </c>
       <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="I6" s="2" t="n"/>
       <c r="J6" s="2" t="n"/>
       <c r="K6" s="2" t="n"/>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="L6" s="2" t="n"/>
       <c r="M6" s="2" t="n"/>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>includes sub-classes for natural disaster, technological disaster, transportation disaster (and each of those has multiple sub-classes)</t>
-        </is>
-      </c>
+      <c r="N6" s="2" t="n"/>
       <c r="O6" s="2" t="n"/>
       <c r="P6" s="2" t="n"/>
       <c r="Q6" s="2" t="inlineStr">
@@ -782,32 +786,32 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
+          <t>potentially traumatic experience</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
           <t>A &lt;potentially traumatic experience&gt; that involves being forced to provide labor against one's will</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience</t>
-        </is>
-      </c>
       <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>includes sub-classes for slavery, human trafficking</t>
+        </is>
+      </c>
       <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="I7" s="2" t="n"/>
       <c r="J7" s="2" t="n"/>
       <c r="K7" s="2" t="n"/>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="L7" s="2" t="n"/>
       <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>includes sub-classes for slavery, human trafficking</t>
-        </is>
-      </c>
+      <c r="N7" s="2" t="n"/>
       <c r="O7" s="2" t="n"/>
       <c r="P7" s="2" t="n"/>
       <c r="Q7" s="2" t="inlineStr">
@@ -831,32 +835,32 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
+          <t>potentially traumatic experience</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
           <t>A &lt;potentially traumatic experience&gt; of some health-related event or treatment.</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience</t>
-        </is>
-      </c>
       <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>includes sub-classes for injury, illness, treatment experiences (and each of these has sub-classes)</t>
+        </is>
+      </c>
       <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="n"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="I8" s="2" t="n"/>
       <c r="J8" s="2" t="n"/>
       <c r="K8" s="2" t="n"/>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="L8" s="2" t="n"/>
       <c r="M8" s="2" t="n"/>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>includes sub-classes for injury, illness, treatment experiences (and each of these has sub-classes)</t>
-        </is>
-      </c>
+      <c r="N8" s="2" t="n"/>
       <c r="O8" s="2" t="n"/>
       <c r="P8" s="2" t="n"/>
       <c r="Q8" s="2" t="inlineStr">
@@ -880,32 +884,32 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
+          <t>potentially traumatic experience</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
           <t>A &lt;potentially traumatic experience&gt; that involves being held against one's will by a government or other state actor</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience</t>
-        </is>
-      </c>
       <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">includes sub-classes for incarceration related to crime, concentration camp imprisonment, political imprisonment, war imprisonment </t>
+        </is>
+      </c>
       <c r="G9" s="2" t="n"/>
-      <c r="H9" s="2" t="n"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="I9" s="2" t="n"/>
       <c r="J9" s="2" t="n"/>
       <c r="K9" s="2" t="n"/>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="L9" s="2" t="n"/>
       <c r="M9" s="2" t="n"/>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">includes sub-classes for incarceration related to crime, concentration camp imprisonment, political imprisonment, war imprisonment </t>
-        </is>
-      </c>
+      <c r="N9" s="2" t="n"/>
       <c r="O9" s="2" t="n"/>
       <c r="P9" s="2" t="n"/>
       <c r="Q9" s="2" t="inlineStr">
@@ -929,32 +933,32 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
+          <t>potentially traumatic experience</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
           <t>A &lt;potentially traumatic experience&gt; that involves abuse that occurs in a familial or caretaking relationship and that may include physical violence</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience</t>
-        </is>
-      </c>
       <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>includes sub-classes: child physical abuse, child sexual abuse, intimate partner violence, elder abuse</t>
+        </is>
+      </c>
       <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="n"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="I10" s="2" t="n"/>
       <c r="J10" s="2" t="n"/>
       <c r="K10" s="2" t="n"/>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="L10" s="2" t="n"/>
       <c r="M10" s="2" t="n"/>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>includes sub-classes: child physical abuse, child sexual abuse, intimate partner violence, elder abuse</t>
-        </is>
-      </c>
+      <c r="N10" s="2" t="n"/>
       <c r="O10" s="2" t="n"/>
       <c r="P10" s="2" t="n"/>
       <c r="Q10" s="2" t="inlineStr">
@@ -978,32 +982,32 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
+          <t>potentially traumatic experience</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
           <t>A &lt;potentially traumatic experience&gt; that involves violence directed at an individual by a person outside their household</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience</t>
-        </is>
-      </c>
       <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>includes sub-classes for physical assault, sexual assault, homicide, abduction-kidnapping, hostage taking, torture</t>
+        </is>
+      </c>
       <c r="G11" s="2" t="n"/>
-      <c r="H11" s="2" t="n"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="I11" s="2" t="n"/>
       <c r="J11" s="2" t="n"/>
       <c r="K11" s="2" t="n"/>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="L11" s="2" t="n"/>
       <c r="M11" s="2" t="n"/>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>includes sub-classes for physical assault, sexual assault, homicide, abduction-kidnapping, hostage taking, torture</t>
-        </is>
-      </c>
+      <c r="N11" s="2" t="n"/>
       <c r="O11" s="2" t="n"/>
       <c r="P11" s="2" t="n"/>
       <c r="Q11" s="2" t="inlineStr">
@@ -1027,32 +1031,32 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
+          <t>potentially traumatic experience</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
           <t>A &lt;potentially traumatic experience&gt; that involves violence directed at a group of people</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience</t>
-        </is>
-      </c>
       <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>includes sub-classes for mass injury or homicide, terrorism, genocide</t>
+        </is>
+      </c>
       <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="n"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="I12" s="2" t="n"/>
       <c r="J12" s="2" t="n"/>
       <c r="K12" s="2" t="n"/>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="L12" s="2" t="n"/>
       <c r="M12" s="2" t="n"/>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>includes sub-classes for mass injury or homicide, terrorism, genocide</t>
-        </is>
-      </c>
+      <c r="N12" s="2" t="n"/>
       <c r="O12" s="2" t="n"/>
       <c r="P12" s="2" t="n"/>
       <c r="Q12" s="2" t="inlineStr">
@@ -1076,32 +1080,32 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
+          <t>potentially traumatic experience</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
           <t>A &lt;potentially traumatic experience&gt; that involves  sudden or forced displacement from one's home or home area because of physical or political danger</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience</t>
-        </is>
-      </c>
       <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>might include sub-classes for refugee experiences, forced migration, prolonged displacement, climate-related displacement</t>
+        </is>
+      </c>
       <c r="G13" s="2" t="n"/>
-      <c r="H13" s="2" t="n"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="I13" s="2" t="n"/>
       <c r="J13" s="2" t="n"/>
       <c r="K13" s="2" t="n"/>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="L13" s="2" t="n"/>
       <c r="M13" s="2" t="n"/>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>might include sub-classes for refugee experiences, forced migration, prolonged displacement, climate-related displacement</t>
-        </is>
-      </c>
+      <c r="N13" s="2" t="n"/>
       <c r="O13" s="2" t="n"/>
       <c r="P13" s="2" t="n"/>
       <c r="Q13" s="2" t="inlineStr">
@@ -1125,32 +1129,32 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
+          <t>potentially traumatic experience</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
           <t>A &lt;potentially traumatic experience&gt; that involves adverse events related to a person's racial or ethnic identity</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience</t>
-        </is>
-      </c>
       <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>includes sub-classes for experiences of racism, hate crimes, micro-agressions, generational trauma</t>
+        </is>
+      </c>
       <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="n"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="n"/>
       <c r="K14" s="2" t="n"/>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="L14" s="2" t="n"/>
       <c r="M14" s="2" t="n"/>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>includes sub-classes for experiences of racism, hate crimes, micro-agressions, generational trauma</t>
-        </is>
-      </c>
+      <c r="N14" s="2" t="n"/>
       <c r="O14" s="2" t="n"/>
       <c r="P14" s="2" t="n"/>
       <c r="Q14" s="2" t="inlineStr">
@@ -1174,32 +1178,32 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
+          <t>potentially traumatic experience</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
           <t>A &lt;potentially traumatic experience&gt; that involves exposure to violence or threat of violence in the social and physical environment outside the person's household.</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience</t>
-        </is>
-      </c>
       <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">includes sub-classes for community evironment of violence; school enviroment of violence; workplace enviroment of violence; environment of violence related to gender, ethnicity or other marginalized identity  </t>
+        </is>
+      </c>
       <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="n"/>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="I15" s="2" t="n"/>
       <c r="J15" s="2" t="n"/>
       <c r="K15" s="2" t="n"/>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="L15" s="2" t="n"/>
       <c r="M15" s="2" t="n"/>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">includes sub-classes for community evironment of violence; school enviroment of violence; workplace enviroment of violence; environment of violence related to gender, ethnicity or other marginalized identity  </t>
-        </is>
-      </c>
+      <c r="N15" s="2" t="n"/>
       <c r="O15" s="2" t="n"/>
       <c r="P15" s="2" t="n"/>
       <c r="Q15" s="2" t="inlineStr">
@@ -1223,15 +1227,15 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
           <t>A process that is the sum of the totality of processes taking place in the spatiotemporal region occupied by a material entity or site, including processes on the surface of the entity or within the cavities to which it serves as host</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>process</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -1250,26 +1254,26 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
           <t>A personal attribute that is the kinship connection of the person a person who has has a specified potentially traumatic experience.</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
         </is>
       </c>
       <c r="E17" s="2" t="n"/>
       <c r="F17" s="2" t="n"/>
       <c r="G17" s="2" t="n"/>
-      <c r="H17" s="2" t="n"/>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="I17" s="2" t="n"/>
       <c r="J17" s="2" t="n"/>
       <c r="K17" s="2" t="n"/>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="L17" s="2" t="n"/>
       <c r="M17" s="2" t="n"/>
       <c r="N17" s="2" t="n"/>
       <c r="O17" s="2" t="n"/>
@@ -1291,26 +1295,26 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
+          <t>potentially traumatic experience severity</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
           <t>The aspect of &lt;potentially traumatic experience severity&gt; that is an objective degree of intensity, damage, or risk</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience severity</t>
         </is>
       </c>
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="n"/>
-      <c r="H18" s="2" t="n"/>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="I18" s="2" t="n"/>
       <c r="J18" s="2" t="n"/>
       <c r="K18" s="2" t="n"/>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="L18" s="2" t="n"/>
       <c r="M18" s="2" t="inlineStr">
         <is>
           <t>dimension</t>
@@ -1336,15 +1340,15 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>entity</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
           <t>An entity that unfolds itself in time or it is the instantaneous boundary of such an entity</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>entity</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -1363,15 +1367,15 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
+          <t>history</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
           <t>A history that is of a person.</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>history</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -1390,15 +1394,15 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
           <t>A process that is part of a personal history.</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>process</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -1417,20 +1421,20 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
+          <t>personal history part</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
           <t>A personal history part that may lead to some traumatic stress response.</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>personal history part</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>Something that a person has experienced that may lead in some cases to some kind of traumatic stress response.</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="n"/>
+      <c r="E22" s="3" t="n"/>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>The use of 'may lead to' is to be interpreted as in at least one case having done so. The focus on 'experience' is designed to recognise that there are other semantic hierarchies for events such as disasters, accidents etc. and that this hierarchy is aimed at classifying the experience of these not the events themselves.</t>
+        </is>
+      </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
           <t>process</t>
@@ -1438,7 +1442,7 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>PTEO</t>
+          <t>Proposed</t>
         </is>
       </c>
       <c r="I22" s="3" t="n"/>
@@ -1446,13 +1450,13 @@
       <c r="K22" s="3" t="n"/>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>PTEO</t>
         </is>
       </c>
       <c r="M22" s="3" t="n"/>
       <c r="N22" s="3" t="inlineStr">
         <is>
-          <t>The use of 'may lead to' is to be interpreted as in at least one case having done so. The focus on 'experience' is designed to recognise that there are other semantic hierarchies for events such as disasters, accidents etc. and that this hierarchy is aimed at classifying the experience of these not the events themselves.</t>
+          <t>Something that a person has experienced that may lead in some cases to some kind of traumatic stress response.</t>
         </is>
       </c>
       <c r="O22" s="3" t="n"/>
@@ -1478,40 +1482,40 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
+          <t>potentially traumatic experience attribute</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
           <t>A &lt;potentially traumatic experience attribute&gt; that is the degree of human agency involved in causing the event(s) experienced</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience attribute</t>
-        </is>
-      </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>The degree to which the causal process involved in the the event(s) which are/were experienced involved human agency / intention to harm.</t>
+          <t>intentionality</t>
         </is>
       </c>
       <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="n"/>
-      <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>intentionality</t>
-        </is>
-      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="n"/>
       <c r="J23" s="2" t="n"/>
       <c r="K23" s="2" t="n"/>
-      <c r="L23" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="L23" s="2" t="n"/>
       <c r="M23" s="2" t="inlineStr">
         <is>
           <t>dimension</t>
         </is>
       </c>
-      <c r="N23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>The degree to which the causal process involved in the the event(s) which are/were experienced involved human agency / intention to harm.</t>
+        </is>
+      </c>
       <c r="O23" s="2" t="n"/>
       <c r="P23" s="2" t="n"/>
       <c r="Q23" s="2" t="inlineStr">
@@ -1535,32 +1539,32 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
+          <t>process attribute</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">A characteristic of a potentially traumatic experience </t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>process attribute</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>Attributes of PTEs include their time course, severity, degree of human agency involved in the event, nature of exposure (direct vs indirect)</t>
-        </is>
-      </c>
+      <c r="E24" s="3" t="n"/>
       <c r="F24" s="3" t="n"/>
       <c r="G24" s="3" t="n"/>
-      <c r="H24" s="3" t="n"/>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
       <c r="I24" s="3" t="n"/>
       <c r="J24" s="3" t="n"/>
       <c r="K24" s="3" t="n"/>
-      <c r="L24" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
+      <c r="L24" s="3" t="n"/>
       <c r="M24" s="3" t="n"/>
-      <c r="N24" s="3" t="n"/>
+      <c r="N24" s="3" t="inlineStr">
+        <is>
+          <t>Attributes of PTEs include their time course, severity, degree of human agency involved in the event, nature of exposure (direct vs indirect)</t>
+        </is>
+      </c>
       <c r="O24" s="3" t="n"/>
       <c r="P24" s="3" t="n"/>
       <c r="Q24" s="3" t="inlineStr">
@@ -1584,34 +1588,34 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
+          <t>potentially traumatic experience attribute</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
           <t>A &lt;potentially traumatic experience attribute&gt; that is the severity of the event(s) experienced.</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience attribute</t>
-        </is>
-      </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>The severity of a PTE relates to its degree of intensity, damage, or risk and includes both objective event factors and the subjective experience of the person.</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="n"/>
+          <t>intensity</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Severity might be seen as a combination of several other attributes listed here - but I think we often think of this as an independent dimension.  Should there be sub-classes for obective severity and subjective or perceived severity, or for objective and perceived life threat?   - to be discussed with colleagues</t>
+        </is>
+      </c>
       <c r="G25" s="2" t="n"/>
-      <c r="H25" s="2" t="n"/>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>intensity</t>
-        </is>
-      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="n"/>
       <c r="J25" s="2" t="n"/>
       <c r="K25" s="2" t="n"/>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="L25" s="2" t="n"/>
       <c r="M25" s="2" t="inlineStr">
         <is>
           <t>dimension</t>
@@ -1619,7 +1623,7 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>Severity might be seen as a combination of several other attributes listed here - but I think we often think of this as an independent dimension.  Should there be sub-classes for obective severity and subjective or perceived severity, or for objective and perceived life threat?   - to be discussed with colleagues</t>
+          <t>The severity of a PTE relates to its degree of intensity, damage, or risk and includes both objective event factors and the subjective experience of the person.</t>
         </is>
       </c>
       <c r="O25" s="2" t="n"/>
@@ -1645,36 +1649,36 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
+          <t>potentially traumatic experience attribute</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
           <t>A &lt;potentially traumatic experience attribute&gt; that is the chronicity, duration, and frequency of the event(s) experienced.</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience attribute</t>
-        </is>
-      </c>
       <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>include sub-classes for chronicity, frequency, duration, age at onset</t>
+        </is>
+      </c>
       <c r="G26" s="2" t="n"/>
-      <c r="H26" s="2" t="n"/>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="I26" s="2" t="n"/>
       <c r="J26" s="2" t="n"/>
       <c r="K26" s="2" t="n"/>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="L26" s="2" t="n"/>
       <c r="M26" s="2" t="inlineStr">
         <is>
           <t>dimension</t>
         </is>
       </c>
-      <c r="N26" s="2" t="inlineStr">
-        <is>
-          <t>include sub-classes for chronicity, frequency, duration, age at onset</t>
-        </is>
-      </c>
+      <c r="N26" s="2" t="n"/>
       <c r="O26" s="2" t="n"/>
       <c r="P26" s="2" t="n"/>
       <c r="Q26" s="2" t="inlineStr">
@@ -1698,30 +1702,30 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
+          <t>potentially traumatic experience attribute</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
           <t>An attribute of a potentially traumatic experience that is the type of event(s) experienced by a person.</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience attribute</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="n"/>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>event type</t>
+        </is>
+      </c>
       <c r="F27" s="4" t="n"/>
       <c r="G27" s="4" t="n"/>
-      <c r="H27" s="4" t="n"/>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>event type</t>
-        </is>
-      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="n"/>
       <c r="J27" s="4" t="n"/>
       <c r="K27" s="4" t="n"/>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="L27" s="4" t="n"/>
       <c r="M27" s="4" t="n"/>
       <c r="N27" s="4" t="n"/>
       <c r="O27" s="4" t="n"/>
@@ -1747,15 +1751,15 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
+          <t>occurrent</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
           <t>An occurrent that has temporal proper parts and for some time t.</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>occurrent</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -1774,15 +1778,15 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
+          <t>process profile</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
           <t>A process profile that is an attribute of a process.</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>process profile</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -1801,22 +1805,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
           <t>b is a process_profile =Def. there is some process c such that b process_profile_of c (axiom label in BFO2 Reference: [093-002])</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>process</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n"/>
+      <c r="A31" s="2" t="inlineStr"/>
       <c r="B31" s="2" t="inlineStr">
         <is>
           <t>subjective severity of potentially traumatic experience</t>
@@ -1824,26 +1828,26 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
+          <t>potentially traumatic experience severity</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
           <t>The aspect of &lt;potentially traumatic experience severity&gt; that is severity (intensity, damage, risk) as subjectively experienced by a person</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience severity</t>
         </is>
       </c>
       <c r="E31" s="2" t="n"/>
       <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="n"/>
-      <c r="H31" s="2" t="n"/>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="I31" s="2" t="n"/>
       <c r="J31" s="2" t="n"/>
       <c r="K31" s="2" t="n"/>
-      <c r="L31" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="L31" s="2" t="n"/>
       <c r="M31" s="2" t="inlineStr">
         <is>
           <t>dimension</t>

</xml_diff>

<commit_message>
Update 2 terms in TSO classes.xlsx
</commit_message>
<xml_diff>
--- a/TSO classes.xlsx
+++ b/TSO classes.xlsx
@@ -725,11 +725,7 @@
       <c r="S5" s="3" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>_:vis-5</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="inlineStr"/>
       <c r="B6" s="2" t="inlineStr">
         <is>
           <t>experience of disaster</t>
@@ -742,7 +738,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves a sudden-onset occurrence created by natural or technological forces impacting a group of people defined by place or region</t>
+          <t>A &lt;potentially traumatic experience&gt; that involves a sudden-onset occurrence created by natural or technological forces impacting a group of people defined by place or region.</t>
         </is>
       </c>
       <c r="E6" s="2" t="n"/>
@@ -1820,7 +1816,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr"/>
+      <c r="A31" s="2" t="n"/>
       <c r="B31" s="2" t="inlineStr">
         <is>
           <t>subjective severity of potentially traumatic experience</t>
@@ -1833,10 +1829,10 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>The aspect of &lt;potentially traumatic experience severity&gt; that is severity (intensity, damage, risk) as subjectively experienced by a person</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="n"/>
+          <t>&lt;Potentially traumatic experience severity&gt; that is subjectively experienced by a person.</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="n"/>
       <c r="H31" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update potentially traumatic experience in TSO classes.xlsx
</commit_message>
<xml_diff>
--- a/TSO classes.xlsx
+++ b/TSO classes.xlsx
@@ -594,7 +594,7 @@
           <t>A &lt;potentially traumatic experience&gt; that involves actual (or potential) injury, without human intention to cause harm, and impacts one or a few people.</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n"/>
+      <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>includes sub-classes for road traffic accident, fall, animal attack, residential fire, sports-related, weapon-related (unintentional), choking, drowning</t>
@@ -725,7 +725,7 @@
       <c r="S5" s="3" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
+      <c r="A6" s="2" t="n"/>
       <c r="B6" s="2" t="inlineStr">
         <is>
           <t>experience of disaster</t>
@@ -1422,10 +1422,10 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>A personal history part that may lead to some traumatic stress response.</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="n"/>
+          <t>A &lt;personal history part&gt; that may lead to some traumatic stress response.</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="3" t="inlineStr">
         <is>
           <t>The use of 'may lead to' is to be interpreted as in at least one case having done so. The focus on 'experience' is designed to recognise that there are other semantic hierarchies for events such as disasters, accidents etc. and that this hierarchy is aimed at classifying the experience of these not the events themselves.</t>
@@ -1832,7 +1832,7 @@
           <t>&lt;Potentially traumatic experience severity&gt; that is subjectively experienced by a person.</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr"/>
+      <c r="E31" s="2" t="n"/>
       <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="n"/>
       <c r="H31" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update Definition of experience of accident in TSO classes.xlsx
</commit_message>
<xml_diff>
--- a/TSO classes.xlsx
+++ b/TSO classes.xlsx
@@ -591,10 +591,10 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves actual (or potential) injury, without human intention to cause harm, and impacts one or a few people.</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr"/>
+          <t>A &lt;potentially traumatic experience&gt; that involves actual harm or the perception of potential harm, without human intention to cause harm and that impacts on one or a few people.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>includes sub-classes for road traffic accident, fall, animal attack, residential fire, sports-related, weapon-related (unintentional), choking, drowning</t>
@@ -1425,7 +1425,7 @@
           <t>A &lt;personal history part&gt; that may lead to some traumatic stress response.</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="n"/>
       <c r="F22" s="3" t="inlineStr">
         <is>
           <t>The use of 'may lead to' is to be interpreted as in at least one case having done so. The focus on 'experience' is designed to recognise that there are other semantic hierarchies for events such as disasters, accidents etc. and that this hierarchy is aimed at classifying the experience of these not the events themselves.</t>

</xml_diff>

<commit_message>
Update experience of military conflict in TSO classes.xlsx
</commit_message>
<xml_diff>
--- a/TSO classes.xlsx
+++ b/TSO classes.xlsx
@@ -627,124 +627,124 @@
       <c r="S3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>TSTO:0000013</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>experience of armed conflict</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>TSTO:0000024</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">experience of bereavement </t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves armed conflict between states or other military groups.</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>includes sub-classes for civilian exposure to warfare or armed conflict, combat exposure as a member of armed forces, deployment as a member of armed forces</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;potentially traumatic experience&gt; that is the death of a loved one.</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="n"/>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>need to consult with colleages about sub-classes - probably traumatic bereavement and others</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="n"/>
+      <c r="M4" s="3" t="n"/>
+      <c r="N4" s="3" t="n"/>
+      <c r="O4" s="3" t="n"/>
+      <c r="P4" s="3" t="n"/>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>NKA</t>
+        </is>
+      </c>
+      <c r="R4" s="3" t="n"/>
+      <c r="S4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n"/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>experience of disaster</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>potentially traumatic experience</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;potentially traumatic experience&gt; that involves a sudden-onset occurrence created by natural or technological forces impacting a group of people defined by place or region.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>includes sub-classes for natural disaster, technological disaster, transportation disaster (and each of those has multiple sub-classes)</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Pre-proposed</t>
         </is>
       </c>
-      <c r="I4" s="2" t="n"/>
-      <c r="J4" s="2" t="n"/>
-      <c r="K4" s="2" t="n"/>
-      <c r="L4" s="2" t="n"/>
-      <c r="M4" s="2" t="n"/>
-      <c r="N4" s="2" t="n"/>
-      <c r="O4" s="2" t="n"/>
-      <c r="P4" s="2" t="n"/>
-      <c r="Q4" s="2" t="inlineStr">
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="n"/>
+      <c r="K5" s="2" t="n"/>
+      <c r="L5" s="2" t="n"/>
+      <c r="M5" s="2" t="n"/>
+      <c r="N5" s="2" t="n"/>
+      <c r="O5" s="2" t="n"/>
+      <c r="P5" s="2" t="n"/>
+      <c r="Q5" s="2" t="inlineStr">
         <is>
           <t>NKA</t>
         </is>
       </c>
-      <c r="R4" s="2" t="n"/>
-      <c r="S4" s="2" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>TSTO:0000024</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">experience of bereavement </t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="R5" s="2" t="n"/>
+      <c r="S5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TSTO:0000004</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>experience of forced labor</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that is the death of a loved one.</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>need to consult with colleages about sub-classes - probably traumatic bereavement and others</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="n"/>
-      <c r="K5" s="3" t="n"/>
-      <c r="L5" s="3" t="n"/>
-      <c r="M5" s="3" t="n"/>
-      <c r="N5" s="3" t="n"/>
-      <c r="O5" s="3" t="n"/>
-      <c r="P5" s="3" t="n"/>
-      <c r="Q5" s="3" t="inlineStr">
-        <is>
-          <t>NKA</t>
-        </is>
-      </c>
-      <c r="R5" s="3" t="n"/>
-      <c r="S5" s="3" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>experience of disaster</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience</t>
-        </is>
-      </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves a sudden-onset occurrence created by natural or technological forces impacting a group of people defined by place or region.</t>
+          <t>A &lt;potentially traumatic experience&gt; that involves being forced to provide labor against one's will</t>
         </is>
       </c>
       <c r="E6" s="2" t="n"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>includes sub-classes for natural disaster, technological disaster, transportation disaster (and each of those has multiple sub-classes)</t>
+          <t>includes sub-classes for slavery, human trafficking</t>
         </is>
       </c>
       <c r="G6" s="2" t="n"/>
@@ -772,12 +772,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>TSTO:0000004</t>
+          <t>TSTO:0000005</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>experience of forced labor</t>
+          <t>experience of health event</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -787,13 +787,13 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves being forced to provide labor against one's will</t>
+          <t>A &lt;potentially traumatic experience&gt; of some health-related event or treatment.</t>
         </is>
       </c>
       <c r="E7" s="2" t="n"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>includes sub-classes for slavery, human trafficking</t>
+          <t>includes sub-classes for injury, illness, treatment experiences (and each of these has sub-classes)</t>
         </is>
       </c>
       <c r="G7" s="2" t="n"/>
@@ -821,12 +821,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TSTO:0000005</t>
+          <t>TSTO:0000006</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>experience of health event</t>
+          <t>experience of incarceration</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -836,13 +836,13 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; of some health-related event or treatment.</t>
+          <t>A &lt;potentially traumatic experience&gt; that involves being held against one's will by a government or other state actor</t>
         </is>
       </c>
       <c r="E8" s="2" t="n"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>includes sub-classes for injury, illness, treatment experiences (and each of these has sub-classes)</t>
+          <t xml:space="preserve">includes sub-classes for incarceration related to crime, concentration camp imprisonment, political imprisonment, war imprisonment </t>
         </is>
       </c>
       <c r="G8" s="2" t="n"/>
@@ -870,12 +870,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>TSTO:0000006</t>
+          <t>TSTO:0000007</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>experience of incarceration</t>
+          <t>experience of interpersonal abuse</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -885,13 +885,13 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves being held against one's will by a government or other state actor</t>
+          <t>A &lt;potentially traumatic experience&gt; that involves abuse that occurs in a familial or caretaking relationship and that may include physical violence</t>
         </is>
       </c>
       <c r="E9" s="2" t="n"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">includes sub-classes for incarceration related to crime, concentration camp imprisonment, political imprisonment, war imprisonment </t>
+          <t>includes sub-classes: child physical abuse, child sexual abuse, intimate partner violence, elder abuse</t>
         </is>
       </c>
       <c r="G9" s="2" t="n"/>
@@ -919,12 +919,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>TSTO:0000007</t>
+          <t>TSTO:0000008</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>experience of interpersonal abuse</t>
+          <t>experience of interpersonal violence outside the household</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -934,13 +934,13 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves abuse that occurs in a familial or caretaking relationship and that may include physical violence</t>
+          <t>A &lt;potentially traumatic experience&gt; that involves violence directed at an individual by a person outside their household</t>
         </is>
       </c>
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>includes sub-classes: child physical abuse, child sexual abuse, intimate partner violence, elder abuse</t>
+          <t>includes sub-classes for physical assault, sexual assault, homicide, abduction-kidnapping, hostage taking, torture</t>
         </is>
       </c>
       <c r="G10" s="2" t="n"/>
@@ -968,12 +968,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>TSTO:0000008</t>
+          <t>TSTO:0000009</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>experience of interpersonal violence outside the household</t>
+          <t>experience of mass violence</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -983,13 +983,13 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves violence directed at an individual by a person outside their household</t>
+          <t>A &lt;potentially traumatic experience&gt; that involves violence directed at a group of people</t>
         </is>
       </c>
       <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>includes sub-classes for physical assault, sexual assault, homicide, abduction-kidnapping, hostage taking, torture</t>
+          <t>includes sub-classes for mass injury or homicide, terrorism, genocide</t>
         </is>
       </c>
       <c r="G11" s="2" t="n"/>
@@ -1017,12 +1017,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>TSTO:0000009</t>
+          <t>TSTO:0000010</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>experience of mass violence</t>
+          <t>experience of migration or displacement</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1032,13 +1032,13 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves violence directed at a group of people</t>
+          <t>A &lt;potentially traumatic experience&gt; that involves  sudden or forced displacement from one's home or home area because of physical or political danger</t>
         </is>
       </c>
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>includes sub-classes for mass injury or homicide, terrorism, genocide</t>
+          <t>might include sub-classes for refugee experiences, forced migration, prolonged displacement, climate-related displacement</t>
         </is>
       </c>
       <c r="G12" s="2" t="n"/>
@@ -1064,53 +1064,53 @@
       <c r="S12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>TSTO:0000010</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>experience of migration or displacement</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>TSTO:0000025</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>experience of military conflict</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves  sudden or forced displacement from one's home or home area because of physical or political danger</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>might include sub-classes for refugee experiences, forced migration, prolonged displacement, climate-related displacement</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="n"/>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="n"/>
-      <c r="J13" s="2" t="n"/>
-      <c r="K13" s="2" t="n"/>
-      <c r="L13" s="2" t="n"/>
-      <c r="M13" s="2" t="n"/>
-      <c r="N13" s="2" t="n"/>
-      <c r="O13" s="2" t="n"/>
-      <c r="P13" s="2" t="n"/>
-      <c r="Q13" s="2" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;potentially traumatic experience&gt; that occurs during or in direct consequence of organised armed conflict.</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>includes sub-classes for civilian exposure to warfare or armed conflict, combat exposure as a member of armed forces, deployment as a member of armed forces</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="n"/>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="n"/>
+      <c r="J13" s="3" t="n"/>
+      <c r="K13" s="3" t="n"/>
+      <c r="L13" s="3" t="n"/>
+      <c r="M13" s="3" t="n"/>
+      <c r="N13" s="3" t="n"/>
+      <c r="O13" s="3" t="n"/>
+      <c r="P13" s="3" t="n"/>
+      <c r="Q13" s="3" t="inlineStr">
         <is>
           <t>NKA</t>
         </is>
       </c>
-      <c r="R13" s="2" t="n"/>
-      <c r="S13" s="2" t="n"/>
+      <c r="R13" s="3" t="n"/>
+      <c r="S13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update experience of bereavement  in TSO classes.xlsx
</commit_message>
<xml_diff>
--- a/TSO classes.xlsx
+++ b/TSO classes.xlsx
@@ -644,13 +644,13 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that is the death of a loved one.</t>
+          <t>A &lt;potentially traumatic experience&gt; that involves the death of a loved one.</t>
         </is>
       </c>
       <c r="E4" s="3" t="n"/>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>need to consult with colleages about sub-classes - probably traumatic bereavement and others</t>
+          <t>need to consult with colleages about sub-classes - probably traumatic bereavement and others but concept of loved one seems to involve close attachment and need not involve positive affection</t>
         </is>
       </c>
       <c r="G4" s="3" t="n"/>
@@ -1084,7 +1084,7 @@
           <t>A &lt;potentially traumatic experience&gt; that occurs during or in direct consequence of organised armed conflict.</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="n"/>
       <c r="F13" s="3" t="inlineStr">
         <is>
           <t>includes sub-classes for civilian exposure to warfare or armed conflict, combat exposure as a member of armed forces, deployment as a member of armed forces</t>

</xml_diff>

<commit_message>
Update Definition of experience of disaster in TSO classes.xlsx
</commit_message>
<xml_diff>
--- a/TSO classes.xlsx
+++ b/TSO classes.xlsx
@@ -689,10 +689,10 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves a sudden-onset occurrence created by natural or technological forces impacting a group of people defined by place or region.</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="n"/>
+          <t>A &lt;potentially traumatic experience&gt; that occurs during or in direct consequence of a discrete catastrophic event or series of events — whether of natural or technological origin — that causes or threatens widespread death, serious injury, destruction of property, or severe disruption to community functioning.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
           <t>includes sub-classes for natural disaster, technological disaster, transportation disaster (and each of those has multiple sub-classes)</t>

</xml_diff>

<commit_message>
Update experience of health-related event in TSO classes.xlsx
</commit_message>
<xml_diff>
--- a/TSO classes.xlsx
+++ b/TSO classes.xlsx
@@ -692,7 +692,7 @@
           <t>A &lt;potentially traumatic experience&gt; that occurs during or in direct consequence of a discrete catastrophic event or series of events — whether of natural or technological origin — that causes or threatens widespread death, serious injury, destruction of property, or severe disruption to community functioning.</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="n"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
           <t>includes sub-classes for natural disaster, technological disaster, transportation disaster (and each of those has multiple sub-classes)</t>
@@ -770,53 +770,53 @@
       <c r="S6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>TSTO:0000005</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>experience of health event</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>experience of health-related event</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; of some health-related event or treatment.</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;potentially traumatic experience&gt; that involves  illness, injury or treatment.</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>includes sub-classes for injury, illness, treatment experiences (and each of these has sub-classes)</t>
         </is>
       </c>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="n"/>
-      <c r="K7" s="2" t="n"/>
-      <c r="L7" s="2" t="n"/>
-      <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="n"/>
-      <c r="O7" s="2" t="n"/>
-      <c r="P7" s="2" t="n"/>
-      <c r="Q7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="n"/>
+      <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n"/>
+      <c r="M7" s="3" t="n"/>
+      <c r="N7" s="3" t="n"/>
+      <c r="O7" s="3" t="n"/>
+      <c r="P7" s="3" t="n"/>
+      <c r="Q7" s="3" t="inlineStr">
         <is>
           <t>NKA</t>
         </is>
       </c>
-      <c r="R7" s="2" t="n"/>
-      <c r="S7" s="2" t="n"/>
+      <c r="R7" s="3" t="n"/>
+      <c r="S7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update experience of state-sanctioned incarceration in TSO classes.xlsx
</commit_message>
<xml_diff>
--- a/TSO classes.xlsx
+++ b/TSO classes.xlsx
@@ -790,7 +790,7 @@
           <t>A &lt;potentially traumatic experience&gt; that involves  illness, injury or treatment.</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="n"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
           <t>includes sub-classes for injury, illness, treatment experiences (and each of these has sub-classes)</t>
@@ -821,12 +821,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TSTO:0000006</t>
+          <t>TSTO:0000007</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>experience of incarceration</t>
+          <t>experience of interpersonal abuse</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -836,13 +836,13 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves being held against one's will by a government or other state actor</t>
+          <t>A &lt;potentially traumatic experience&gt; that involves abuse that occurs in a familial or caretaking relationship and that may include physical violence</t>
         </is>
       </c>
       <c r="E8" s="2" t="n"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">includes sub-classes for incarceration related to crime, concentration camp imprisonment, political imprisonment, war imprisonment </t>
+          <t>includes sub-classes: child physical abuse, child sexual abuse, intimate partner violence, elder abuse</t>
         </is>
       </c>
       <c r="G8" s="2" t="n"/>
@@ -870,12 +870,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>TSTO:0000007</t>
+          <t>TSTO:0000008</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>experience of interpersonal abuse</t>
+          <t>experience of interpersonal violence outside the household</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -885,13 +885,13 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves abuse that occurs in a familial or caretaking relationship and that may include physical violence</t>
+          <t>A &lt;potentially traumatic experience&gt; that involves violence directed at an individual by a person outside their household</t>
         </is>
       </c>
       <c r="E9" s="2" t="n"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>includes sub-classes: child physical abuse, child sexual abuse, intimate partner violence, elder abuse</t>
+          <t>includes sub-classes for physical assault, sexual assault, homicide, abduction-kidnapping, hostage taking, torture</t>
         </is>
       </c>
       <c r="G9" s="2" t="n"/>
@@ -919,12 +919,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>TSTO:0000008</t>
+          <t>TSTO:0000009</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>experience of interpersonal violence outside the household</t>
+          <t>experience of mass violence</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -934,13 +934,13 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves violence directed at an individual by a person outside their household</t>
+          <t>A &lt;potentially traumatic experience&gt; that involves violence directed at a group of people</t>
         </is>
       </c>
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>includes sub-classes for physical assault, sexual assault, homicide, abduction-kidnapping, hostage taking, torture</t>
+          <t>includes sub-classes for mass injury or homicide, terrorism, genocide</t>
         </is>
       </c>
       <c r="G10" s="2" t="n"/>
@@ -968,12 +968,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>TSTO:0000009</t>
+          <t>TSTO:0000010</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>experience of mass violence</t>
+          <t>experience of migration or displacement</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -983,13 +983,13 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves violence directed at a group of people</t>
+          <t>A &lt;potentially traumatic experience&gt; that involves  sudden or forced displacement from one's home or home area because of physical or political danger</t>
         </is>
       </c>
       <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>includes sub-classes for mass injury or homicide, terrorism, genocide</t>
+          <t>might include sub-classes for refugee experiences, forced migration, prolonged displacement, climate-related displacement</t>
         </is>
       </c>
       <c r="G11" s="2" t="n"/>
@@ -1015,151 +1015,151 @@
       <c r="S11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>TSTO:0000010</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>experience of migration or displacement</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>TSTO:0000025</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>experience of military conflict</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves  sudden or forced displacement from one's home or home area because of physical or political danger</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>might include sub-classes for refugee experiences, forced migration, prolonged displacement, climate-related displacement</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;potentially traumatic experience&gt; that occurs during or in direct consequence of organised armed conflict.</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>includes sub-classes for civilian exposure to warfare or armed conflict, combat exposure as a member of armed forces, deployment as a member of armed forces</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="n"/>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="n"/>
+      <c r="J12" s="3" t="n"/>
+      <c r="K12" s="3" t="n"/>
+      <c r="L12" s="3" t="n"/>
+      <c r="M12" s="3" t="n"/>
+      <c r="N12" s="3" t="n"/>
+      <c r="O12" s="3" t="n"/>
+      <c r="P12" s="3" t="n"/>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>NKA</t>
+        </is>
+      </c>
+      <c r="R12" s="3" t="n"/>
+      <c r="S12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TSTO:0000011</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>experience of racial trauma</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>potentially traumatic experience</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;potentially traumatic experience&gt; that involves adverse events related to a person's racial or ethnic identity</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>includes sub-classes for experiences of racism, hate crimes, micro-agressions, generational trauma</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Pre-proposed</t>
         </is>
       </c>
-      <c r="I12" s="2" t="n"/>
-      <c r="J12" s="2" t="n"/>
-      <c r="K12" s="2" t="n"/>
-      <c r="L12" s="2" t="n"/>
-      <c r="M12" s="2" t="n"/>
-      <c r="N12" s="2" t="n"/>
-      <c r="O12" s="2" t="n"/>
-      <c r="P12" s="2" t="n"/>
-      <c r="Q12" s="2" t="inlineStr">
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="n"/>
+      <c r="K13" s="2" t="n"/>
+      <c r="L13" s="2" t="n"/>
+      <c r="M13" s="2" t="n"/>
+      <c r="N13" s="2" t="n"/>
+      <c r="O13" s="2" t="n"/>
+      <c r="P13" s="2" t="n"/>
+      <c r="Q13" s="2" t="inlineStr">
         <is>
           <t>NKA</t>
         </is>
       </c>
-      <c r="R12" s="2" t="n"/>
-      <c r="S12" s="2" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>TSTO:0000025</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>experience of military conflict</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="R13" s="2" t="n"/>
+      <c r="S13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>TSTO:0000006</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>experience of state-sanctioned incarceration</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that occurs during or in direct consequence of organised armed conflict.</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="n"/>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>includes sub-classes for civilian exposure to warfare or armed conflict, combat exposure as a member of armed forces, deployment as a member of armed forces</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="n"/>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;potentially traumatic experience&gt; that involves being confined by a state or state-sanctioned authority.</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n"/>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">includes sub-classes for incarceration related to crime, concentration camp imprisonment, political imprisonment, war imprisonment </t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr"/>
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="I13" s="3" t="n"/>
-      <c r="J13" s="3" t="n"/>
-      <c r="K13" s="3" t="n"/>
-      <c r="L13" s="3" t="n"/>
-      <c r="M13" s="3" t="n"/>
-      <c r="N13" s="3" t="n"/>
-      <c r="O13" s="3" t="n"/>
-      <c r="P13" s="3" t="n"/>
-      <c r="Q13" s="3" t="inlineStr">
+      <c r="I14" s="3" t="n"/>
+      <c r="J14" s="3" t="n"/>
+      <c r="K14" s="3" t="n"/>
+      <c r="L14" s="3" t="n"/>
+      <c r="M14" s="3" t="n"/>
+      <c r="N14" s="3" t="n"/>
+      <c r="O14" s="3" t="n"/>
+      <c r="P14" s="3" t="n"/>
+      <c r="Q14" s="3" t="inlineStr">
         <is>
           <t>NKA</t>
         </is>
       </c>
-      <c r="R13" s="3" t="n"/>
-      <c r="S13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>TSTO:0000011</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>experience of racial trauma</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves adverse events related to a person's racial or ethnic identity</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>includes sub-classes for experiences of racism, hate crimes, micro-agressions, generational trauma</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="n"/>
-      <c r="J14" s="2" t="n"/>
-      <c r="K14" s="2" t="n"/>
-      <c r="L14" s="2" t="n"/>
-      <c r="M14" s="2" t="n"/>
-      <c r="N14" s="2" t="n"/>
-      <c r="O14" s="2" t="n"/>
-      <c r="P14" s="2" t="n"/>
-      <c r="Q14" s="2" t="inlineStr">
-        <is>
-          <t>NKA</t>
-        </is>
-      </c>
-      <c r="R14" s="2" t="n"/>
-      <c r="S14" s="2" t="n"/>
+      <c r="R14" s="3" t="n"/>
+      <c r="S14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update experience of displacement in TSO classes.xlsx
</commit_message>
<xml_diff>
--- a/TSO classes.xlsx
+++ b/TSO classes.xlsx
@@ -723,12 +723,12 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>TSTO:0000007</t>
+          <t>TSTO:0000010</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>experience of familial interpersonal abuse</t>
+          <t>experience of displacement</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -738,13 +738,13 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves repeated abuse that occurs between people in a familial or caretaking relationship.</t>
+          <t>A &lt;potentially traumatic experience&gt; that involves  displacement from the person's home area because of physical or political danger or by force.</t>
         </is>
       </c>
       <c r="E6" s="3" t="n"/>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>includes sub-classes: child physical abuse, child sexual abuse, intimate partner violence, elder abuse</t>
+          <t>might include sub-classes for refugee experiences, forced migration, prolonged displacement, climate-related displacement</t>
         </is>
       </c>
       <c r="G6" s="3" t="n"/>
@@ -770,112 +770,112 @@
       <c r="S6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>TSTO:0000007</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>experience of familial interpersonal abuse</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>potentially traumatic experience</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;potentially traumatic experience&gt; that involves repeated abuse that occurs between people in a familial or caretaking relationship.</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>includes sub-classes: child physical abuse, child sexual abuse, intimate partner violence, elder abuse</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="n"/>
+      <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n"/>
+      <c r="M7" s="3" t="n"/>
+      <c r="N7" s="3" t="n"/>
+      <c r="O7" s="3" t="n"/>
+      <c r="P7" s="3" t="n"/>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>NKA</t>
+        </is>
+      </c>
+      <c r="R7" s="3" t="n"/>
+      <c r="S7" s="3" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>TSTO:0000004</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>experience of forced labor</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>A &lt;potentially traumatic experience&gt; that involves the person being compelled to provide labor through force, threat, deception, or abuse of power, and without the possibility of free and informed refusal</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>includes sub-classes for slavery, human trafficking</t>
         </is>
       </c>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Pre-proposed</t>
         </is>
       </c>
-      <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="n"/>
-      <c r="K7" s="2" t="n"/>
-      <c r="L7" s="2" t="n"/>
-      <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="n"/>
-      <c r="O7" s="2" t="n"/>
-      <c r="P7" s="2" t="n"/>
-      <c r="Q7" s="2" t="inlineStr">
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" s="2" t="n"/>
+      <c r="K8" s="2" t="n"/>
+      <c r="L8" s="2" t="n"/>
+      <c r="M8" s="2" t="n"/>
+      <c r="N8" s="2" t="n"/>
+      <c r="O8" s="2" t="n"/>
+      <c r="P8" s="2" t="n"/>
+      <c r="Q8" s="2" t="inlineStr">
         <is>
           <t>NKA</t>
         </is>
       </c>
-      <c r="R7" s="2" t="n"/>
-      <c r="S7" s="2" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>TSTO:0000005</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>experience of health-related event</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves  illness, injury or treatment.</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>includes sub-classes for injury, illness, treatment experiences (and each of these has sub-classes)</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="n"/>
-      <c r="J8" s="3" t="n"/>
-      <c r="K8" s="3" t="n"/>
-      <c r="L8" s="3" t="n"/>
-      <c r="M8" s="3" t="n"/>
-      <c r="N8" s="3" t="n"/>
-      <c r="O8" s="3" t="n"/>
-      <c r="P8" s="3" t="n"/>
-      <c r="Q8" s="3" t="inlineStr">
-        <is>
-          <t>NKA</t>
-        </is>
-      </c>
-      <c r="R8" s="3" t="n"/>
-      <c r="S8" s="3" t="n"/>
+      <c r="R8" s="2" t="n"/>
+      <c r="S8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>TSTO:0000008</t>
+          <t>TSTO:0000005</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>experience of interpersonal violence</t>
+          <t>experience of health-related event</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -885,13 +885,13 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves violence perpetrated by one or more other persons, outside of the context of organised armed conflict.</t>
+          <t>A &lt;potentially traumatic experience&gt; that involves  illness, injury or treatment.</t>
         </is>
       </c>
       <c r="E9" s="3" t="n"/>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>includes sub-classes for physical assault, sexual assault, homicide, abduction-kidnapping, hostage taking, torture</t>
+          <t>includes sub-classes for injury, illness, treatment experiences (and each of these has sub-classes)</t>
         </is>
       </c>
       <c r="G9" s="3" t="n"/>
@@ -919,12 +919,12 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>TSTO:0000009</t>
+          <t>TSTO:0000008</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>experience of mass violence</t>
+          <t>experience of interpersonal violence</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -934,13 +934,13 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves experience of violence directed at a group of people.</t>
+          <t>A &lt;potentially traumatic experience&gt; that involves violence perpetrated by one or more other persons, outside of the context of organised armed conflict.</t>
         </is>
       </c>
       <c r="E10" s="3" t="n"/>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>includes sub-classes for mass injury or homicide, terrorism, genocide</t>
+          <t>includes sub-classes for physical assault, sexual assault, homicide, abduction-kidnapping, hostage taking, torture</t>
         </is>
       </c>
       <c r="G10" s="3" t="n"/>
@@ -966,53 +966,53 @@
       <c r="S10" s="3" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>TSTO:0000010</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>experience of migration or displacement</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>TSTO:0000009</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>experience of mass violence</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves  sudden or forced displacement from one's home or home area because of physical or political danger</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>might include sub-classes for refugee experiences, forced migration, prolonged displacement, climate-related displacement</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="n"/>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="n"/>
-      <c r="J11" s="2" t="n"/>
-      <c r="K11" s="2" t="n"/>
-      <c r="L11" s="2" t="n"/>
-      <c r="M11" s="2" t="n"/>
-      <c r="N11" s="2" t="n"/>
-      <c r="O11" s="2" t="n"/>
-      <c r="P11" s="2" t="n"/>
-      <c r="Q11" s="2" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;potentially traumatic experience&gt; that involves experience of violence directed at a group of people.</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="n"/>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>includes sub-classes for mass injury or homicide, terrorism, genocide</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="n"/>
+      <c r="J11" s="3" t="n"/>
+      <c r="K11" s="3" t="n"/>
+      <c r="L11" s="3" t="n"/>
+      <c r="M11" s="3" t="n"/>
+      <c r="N11" s="3" t="n"/>
+      <c r="O11" s="3" t="n"/>
+      <c r="P11" s="3" t="n"/>
+      <c r="Q11" s="3" t="inlineStr">
         <is>
           <t>NKA</t>
         </is>
       </c>
-      <c r="R11" s="2" t="n"/>
-      <c r="S11" s="2" t="n"/>
+      <c r="R11" s="3" t="n"/>
+      <c r="S11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update experience of racial trauma in TSO classes.xlsx
</commit_message>
<xml_diff>
--- a/TSO classes.xlsx
+++ b/TSO classes.xlsx
@@ -1064,53 +1064,53 @@
       <c r="S12" s="3" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>TSTO:0000011</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>experience of racial trauma</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves adverse events related to a person's racial or ethnic identity</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;potentially traumatic experience&gt; that involves adversity or harm related to the person's perceived race or ethnicity or their racial or ethnic identity.</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>includes sub-classes for experiences of racism, hate crimes, micro-agressions, generational trauma</t>
         </is>
       </c>
-      <c r="G13" s="2" t="n"/>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="n"/>
-      <c r="J13" s="2" t="n"/>
-      <c r="K13" s="2" t="n"/>
-      <c r="L13" s="2" t="n"/>
-      <c r="M13" s="2" t="n"/>
-      <c r="N13" s="2" t="n"/>
-      <c r="O13" s="2" t="n"/>
-      <c r="P13" s="2" t="n"/>
-      <c r="Q13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="n"/>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="n"/>
+      <c r="J13" s="3" t="n"/>
+      <c r="K13" s="3" t="n"/>
+      <c r="L13" s="3" t="n"/>
+      <c r="M13" s="3" t="n"/>
+      <c r="N13" s="3" t="n"/>
+      <c r="O13" s="3" t="n"/>
+      <c r="P13" s="3" t="n"/>
+      <c r="Q13" s="3" t="inlineStr">
         <is>
           <t>NKA</t>
         </is>
       </c>
-      <c r="R13" s="2" t="n"/>
-      <c r="S13" s="2" t="n"/>
+      <c r="R13" s="3" t="n"/>
+      <c r="S13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add experience of interpersonal abuse to TSO classes.xlsx
</commit_message>
<xml_diff>
--- a/TSO classes.xlsx
+++ b/TSO classes.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S31"/>
+  <dimension ref="A1:S32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -917,63 +917,51 @@
       <c r="S9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>TSTO:0000008</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>experience of interpersonal violence</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>experience of interpersonal abuse</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves violence perpetrated by one or more other persons, outside of the context of organised armed conflict.</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>includes sub-classes for physical assault, sexual assault, homicide, abduction-kidnapping, hostage taking, torture</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="n"/>
-      <c r="J10" s="3" t="n"/>
-      <c r="K10" s="3" t="n"/>
-      <c r="L10" s="3" t="n"/>
-      <c r="M10" s="3" t="n"/>
-      <c r="N10" s="3" t="n"/>
-      <c r="O10" s="3" t="n"/>
-      <c r="P10" s="3" t="n"/>
-      <c r="Q10" s="3" t="inlineStr">
-        <is>
-          <t>NKA</t>
-        </is>
-      </c>
-      <c r="R10" s="3" t="n"/>
-      <c r="S10" s="3" t="n"/>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;potentially traumatic experience&gt; that involves repeated or sustained harm caused by one or ore other people.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr"/>
+      <c r="P10" s="2" t="inlineStr"/>
+      <c r="Q10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>TSTO:0000009</t>
+          <t>TSTO:0000008</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>experience of mass violence</t>
+          <t>experience of interpersonal violence</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -983,13 +971,13 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves experience of violence directed at a group of people.</t>
+          <t>A &lt;potentially traumatic experience&gt; that involves violence perpetrated by one or more other persons, outside of the context of organised armed conflict.</t>
         </is>
       </c>
       <c r="E11" s="3" t="n"/>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>includes sub-classes for mass injury or homicide, terrorism, genocide</t>
+          <t>includes sub-classes for physical assault, sexual assault, homicide, abduction-kidnapping, hostage taking, torture</t>
         </is>
       </c>
       <c r="G11" s="3" t="n"/>
@@ -1017,12 +1005,12 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>TSTO:0000025</t>
+          <t>TSTO:0000009</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>experience of military conflict</t>
+          <t>experience of mass violence</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1032,13 +1020,13 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that occurs during or in direct consequence of organised armed conflict.</t>
+          <t>A &lt;potentially traumatic experience&gt; that involves experience of violence directed at a group of people.</t>
         </is>
       </c>
       <c r="E12" s="3" t="n"/>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>includes sub-classes for civilian exposure to warfare or armed conflict, combat exposure as a member of armed forces, deployment as a member of armed forces</t>
+          <t>includes sub-classes for mass injury or homicide, terrorism, genocide</t>
         </is>
       </c>
       <c r="G12" s="3" t="n"/>
@@ -1066,12 +1054,12 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>TSTO:0000011</t>
+          <t>TSTO:0000025</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>experience of racial trauma</t>
+          <t>experience of military conflict</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -1081,13 +1069,13 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves adversity or harm related to the person's perceived race or ethnicity or their racial or ethnic identity.</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr"/>
+          <t>A &lt;potentially traumatic experience&gt; that occurs during or in direct consequence of organised armed conflict.</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="n"/>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>includes sub-classes for experiences of racism, hate crimes, micro-agressions, generational trauma</t>
+          <t>includes sub-classes for civilian exposure to warfare or armed conflict, combat exposure as a member of armed forces, deployment as a member of armed forces</t>
         </is>
       </c>
       <c r="G13" s="3" t="n"/>
@@ -1115,12 +1103,12 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>TSTO:0000006</t>
+          <t>TSTO:0000011</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>experience of state-sanctioned incarceration</t>
+          <t>experience of racial trauma</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1130,13 +1118,13 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves being confined by a state or state-sanctioned authority.</t>
+          <t>A &lt;potentially traumatic experience&gt; that involves adversity or harm related to the person's perceived race or ethnicity or their racial or ethnic identity.</t>
         </is>
       </c>
       <c r="E14" s="3" t="n"/>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">includes sub-classes for incarceration related to crime, concentration camp imprisonment, political imprisonment, war imprisonment </t>
+          <t>includes sub-classes for experiences of racism, hate crimes, micro-agressions, generational trauma</t>
         </is>
       </c>
       <c r="G14" s="3" t="n"/>
@@ -1164,12 +1152,12 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>TSTO:0000012</t>
+          <t>TSTO:0000006</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>experience of violent social environment</t>
+          <t>experience of state-sanctioned incarceration</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1179,13 +1167,13 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves ongoing exposure to a social environment in which violence is common.</t>
+          <t>A &lt;potentially traumatic experience&gt; that involves being confined by a state or state-sanctioned authority.</t>
         </is>
       </c>
       <c r="E15" s="3" t="n"/>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">includes sub-classes for community evironment of violence; school enviroment of violence; workplace enviroment of violence; environment of violence related to gender, ethnicity or other marginalized identity  </t>
+          <t xml:space="preserve">includes sub-classes for incarceration related to crime, concentration camp imprisonment, political imprisonment, war imprisonment </t>
         </is>
       </c>
       <c r="G15" s="3" t="n"/>
@@ -1211,92 +1199,100 @@
       <c r="S15" s="3" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>TSTO:0000012</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>experience of violent social environment</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>potentially traumatic experience</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;potentially traumatic experience&gt; that involves ongoing exposure to a social environment in which violence is common.</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n"/>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">includes sub-classes for community evironment of violence; school enviroment of violence; workplace enviroment of violence; environment of violence related to gender, ethnicity or other marginalized identity  </t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="n"/>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="n"/>
+      <c r="J16" s="3" t="n"/>
+      <c r="K16" s="3" t="n"/>
+      <c r="L16" s="3" t="n"/>
+      <c r="M16" s="3" t="n"/>
+      <c r="N16" s="3" t="n"/>
+      <c r="O16" s="3" t="n"/>
+      <c r="P16" s="3" t="n"/>
+      <c r="Q16" s="3" t="inlineStr">
+        <is>
+          <t>NKA</t>
+        </is>
+      </c>
+      <c r="R16" s="3" t="n"/>
+      <c r="S16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>BFO:0000182</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>history</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>A process that is the sum of the totality of processes taking place in the spatiotemporal region occupied by a material entity or site, including processes on the surface of the entity or within the cavities to which it serves as host</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>TSTO:0000022</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>kinship relationship with potentially traumatic experience target</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>A personal attribute that is the kinship connection of the person a person who has has a specified potentially traumatic experience.</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
-      <c r="G17" s="2" t="n"/>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="n"/>
-      <c r="J17" s="2" t="n"/>
-      <c r="K17" s="2" t="n"/>
-      <c r="L17" s="2" t="n"/>
-      <c r="M17" s="2" t="n"/>
-      <c r="N17" s="2" t="n"/>
-      <c r="O17" s="2" t="n"/>
-      <c r="P17" s="2" t="n"/>
-      <c r="Q17" s="2" t="n"/>
-      <c r="R17" s="2" t="n"/>
-      <c r="S17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>TSTO:0000023</t>
+          <t>TSTO:0000022</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>objective severity of potentially traumatic event(s)</t>
+          <t>kinship relationship with potentially traumatic experience target</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>potentially traumatic experience severity</t>
+          <t>personal attribute</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>The aspect of &lt;potentially traumatic experience severity&gt; that is an objective degree of intensity, damage, or risk</t>
+          <t>A personal attribute that is the kinship connection of the person a person who has has a specified potentially traumatic experience.</t>
         </is>
       </c>
       <c r="E18" s="2" t="n"/>
@@ -1311,11 +1307,7 @@
       <c r="J18" s="2" t="n"/>
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="n"/>
-      <c r="M18" s="2" t="inlineStr">
-        <is>
-          <t>dimension</t>
-        </is>
-      </c>
+      <c r="M18" s="2" t="n"/>
       <c r="N18" s="2" t="n"/>
       <c r="O18" s="2" t="n"/>
       <c r="P18" s="2" t="n"/>
@@ -1324,51 +1316,69 @@
       <c r="S18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>BFO:0000003</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>occurrent</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>entity</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>An entity that unfolds itself in time or it is the instantaneous boundary of such an entity</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>TSTO:0000023</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>objective severity of potentially traumatic event(s)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>potentially traumatic experience severity</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>The aspect of &lt;potentially traumatic experience severity&gt; that is an objective degree of intensity, damage, or risk</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="n"/>
+      <c r="J19" s="2" t="n"/>
+      <c r="K19" s="2" t="n"/>
+      <c r="L19" s="2" t="n"/>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>dimension</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="n"/>
+      <c r="O19" s="2" t="n"/>
+      <c r="P19" s="2" t="n"/>
+      <c r="Q19" s="2" t="n"/>
+      <c r="R19" s="2" t="n"/>
+      <c r="S19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BCIO:015161</t>
+          <t>BFO:0000003</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>personal history</t>
+          <t>occurrent</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>history</t>
+          <t>entity</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>A history that is of a person.</t>
+          <t>An entity that unfolds itself in time or it is the instantaneous boundary of such an entity</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1380,267 +1390,233 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>BCIO:015161</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>personal history</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>history</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>A history that is of a person.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>BCIO:050487</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>A process that is part of a personal history.</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>TSTO:0000001</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>A &lt;personal history part&gt; that may lead to some traumatic stress response.</t>
         </is>
       </c>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="E23" s="3" t="n"/>
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>The use of 'may lead to' is to be interpreted as in at least one case having done so. The focus on 'experience' is designed to recognise that there are other semantic hierarchies for events such as disasters, accidents etc. and that this hierarchy is aimed at classifying the experience of these not the events themselves.</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="I22" s="3" t="n"/>
-      <c r="J22" s="3" t="n"/>
-      <c r="K22" s="3" t="n"/>
-      <c r="L22" s="3" t="inlineStr">
+      <c r="I23" s="3" t="n"/>
+      <c r="J23" s="3" t="n"/>
+      <c r="K23" s="3" t="n"/>
+      <c r="L23" s="3" t="inlineStr">
         <is>
           <t>PTEO</t>
         </is>
       </c>
-      <c r="M22" s="3" t="n"/>
-      <c r="N22" s="3" t="inlineStr">
+      <c r="M23" s="3" t="n"/>
+      <c r="N23" s="3" t="inlineStr">
         <is>
           <t>Something that a person has experienced that may lead in some cases to some kind of traumatic stress response.</t>
         </is>
       </c>
-      <c r="O22" s="3" t="n"/>
-      <c r="P22" s="3" t="n"/>
-      <c r="Q22" s="3" t="inlineStr">
+      <c r="O23" s="3" t="n"/>
+      <c r="P23" s="3" t="n"/>
+      <c r="Q23" s="3" t="inlineStr">
         <is>
           <t>NKA</t>
         </is>
       </c>
-      <c r="R22" s="3" t="n"/>
-      <c r="S22" s="3" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="R23" s="3" t="n"/>
+      <c r="S23" s="3" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>TSTO:0000016</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">potentially traumatic experience - degree of human agency </t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>potentially traumatic experience attribute</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>A &lt;potentially traumatic experience attribute&gt; that is the degree of human agency involved in causing the event(s) experienced</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>intentionality</t>
         </is>
       </c>
-      <c r="F23" s="2" t="n"/>
-      <c r="G23" s="2" t="n"/>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>Pre-proposed</t>
         </is>
       </c>
-      <c r="I23" s="2" t="n"/>
-      <c r="J23" s="2" t="n"/>
-      <c r="K23" s="2" t="n"/>
-      <c r="L23" s="2" t="n"/>
-      <c r="M23" s="2" t="inlineStr">
+      <c r="I24" s="2" t="n"/>
+      <c r="J24" s="2" t="n"/>
+      <c r="K24" s="2" t="n"/>
+      <c r="L24" s="2" t="n"/>
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>dimension</t>
         </is>
       </c>
-      <c r="N23" s="2" t="inlineStr">
+      <c r="N24" s="2" t="inlineStr">
         <is>
           <t>The degree to which the causal process involved in the the event(s) which are/were experienced involved human agency / intention to harm.</t>
         </is>
       </c>
-      <c r="O23" s="2" t="n"/>
-      <c r="P23" s="2" t="n"/>
-      <c r="Q23" s="2" t="inlineStr">
+      <c r="O24" s="2" t="n"/>
+      <c r="P24" s="2" t="n"/>
+      <c r="Q24" s="2" t="inlineStr">
         <is>
           <t>NKA</t>
         </is>
       </c>
-      <c r="R23" s="2" t="n"/>
-      <c r="S23" s="2" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="R24" s="2" t="n"/>
+      <c r="S24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>TSTO:0000021</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>potentially traumatic experience attribute</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>process attribute</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">A characteristic of a potentially traumatic experience </t>
         </is>
       </c>
-      <c r="E24" s="3" t="n"/>
-      <c r="F24" s="3" t="n"/>
-      <c r="G24" s="3" t="n"/>
-      <c r="H24" s="3" t="inlineStr">
+      <c r="E25" s="3" t="n"/>
+      <c r="F25" s="3" t="n"/>
+      <c r="G25" s="3" t="n"/>
+      <c r="H25" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="I24" s="3" t="n"/>
-      <c r="J24" s="3" t="n"/>
-      <c r="K24" s="3" t="n"/>
-      <c r="L24" s="3" t="n"/>
-      <c r="M24" s="3" t="n"/>
-      <c r="N24" s="3" t="inlineStr">
+      <c r="I25" s="3" t="n"/>
+      <c r="J25" s="3" t="n"/>
+      <c r="K25" s="3" t="n"/>
+      <c r="L25" s="3" t="n"/>
+      <c r="M25" s="3" t="n"/>
+      <c r="N25" s="3" t="inlineStr">
         <is>
           <t>Attributes of PTEs include their time course, severity, degree of human agency involved in the event, nature of exposure (direct vs indirect)</t>
         </is>
       </c>
-      <c r="O24" s="3" t="n"/>
-      <c r="P24" s="3" t="n"/>
-      <c r="Q24" s="3" t="inlineStr">
+      <c r="O25" s="3" t="n"/>
+      <c r="P25" s="3" t="n"/>
+      <c r="Q25" s="3" t="inlineStr">
         <is>
           <t>NKA</t>
         </is>
       </c>
-      <c r="R24" s="3" t="n"/>
-      <c r="S24" s="3" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>TSTO:0000018</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience severity</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience attribute</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience attribute&gt; that is the severity of the event(s) experienced.</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>intensity</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>Severity might be seen as a combination of several other attributes listed here - but I think we often think of this as an independent dimension.  Should there be sub-classes for obective severity and subjective or perceived severity, or for objective and perceived life threat?   - to be discussed with colleagues</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="n"/>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
-      <c r="I25" s="2" t="n"/>
-      <c r="J25" s="2" t="n"/>
-      <c r="K25" s="2" t="n"/>
-      <c r="L25" s="2" t="n"/>
-      <c r="M25" s="2" t="inlineStr">
-        <is>
-          <t>dimension</t>
-        </is>
-      </c>
-      <c r="N25" s="2" t="inlineStr">
-        <is>
-          <t>The severity of a PTE relates to its degree of intensity, damage, or risk and includes both objective event factors and the subjective experience of the person.</t>
-        </is>
-      </c>
-      <c r="O25" s="2" t="n"/>
-      <c r="P25" s="2" t="n"/>
-      <c r="Q25" s="2" t="inlineStr">
-        <is>
-          <t>NKA</t>
-        </is>
-      </c>
-      <c r="R25" s="2" t="n"/>
-      <c r="S25" s="2" t="n"/>
+      <c r="R25" s="3" t="n"/>
+      <c r="S25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>TSTO:0000019</t>
+          <t>TSTO:0000018</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>potentially traumatic experience time course</t>
+          <t>potentially traumatic experience severity</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1650,13 +1626,17 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience attribute&gt; that is the chronicity, duration, and frequency of the event(s) experienced.</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="n"/>
+          <t>A &lt;potentially traumatic experience attribute&gt; that is the severity of the event(s) experienced.</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>intensity</t>
+        </is>
+      </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>include sub-classes for chronicity, frequency, duration, age at onset</t>
+          <t>Severity might be seen as a combination of several other attributes listed here - but I think we often think of this as an independent dimension.  Should there be sub-classes for obective severity and subjective or perceived severity, or for objective and perceived life threat?   - to be discussed with colleagues</t>
         </is>
       </c>
       <c r="G26" s="2" t="n"/>
@@ -1674,7 +1654,11 @@
           <t>dimension</t>
         </is>
       </c>
-      <c r="N26" s="2" t="n"/>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>The severity of a PTE relates to its degree of intensity, damage, or risk and includes both objective event factors and the subjective experience of the person.</t>
+        </is>
+      </c>
       <c r="O26" s="2" t="n"/>
       <c r="P26" s="2" t="n"/>
       <c r="Q26" s="2" t="inlineStr">
@@ -1686,100 +1670,126 @@
       <c r="S26" s="2" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>TSTO:0000019</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>potentially traumatic experience time course</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>potentially traumatic experience attribute</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;potentially traumatic experience attribute&gt; that is the chronicity, duration, and frequency of the event(s) experienced.</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>include sub-classes for chronicity, frequency, duration, age at onset</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="n"/>
+      <c r="J27" s="2" t="n"/>
+      <c r="K27" s="2" t="n"/>
+      <c r="L27" s="2" t="n"/>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>dimension</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="n"/>
+      <c r="O27" s="2" t="n"/>
+      <c r="P27" s="2" t="n"/>
+      <c r="Q27" s="2" t="inlineStr">
+        <is>
+          <t>NKA</t>
+        </is>
+      </c>
+      <c r="R27" s="2" t="n"/>
+      <c r="S27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>TSTO:0000020</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>potentially traumatic experience type</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>potentially traumatic experience attribute</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>An attribute of a potentially traumatic experience that is the type of event(s) experienced by a person.</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>event type</t>
         </is>
       </c>
-      <c r="F27" s="4" t="n"/>
-      <c r="G27" s="4" t="n"/>
-      <c r="H27" s="4" t="inlineStr">
+      <c r="F28" s="4" t="n"/>
+      <c r="G28" s="4" t="n"/>
+      <c r="H28" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="I27" s="4" t="n"/>
-      <c r="J27" s="4" t="n"/>
-      <c r="K27" s="4" t="n"/>
-      <c r="L27" s="4" t="n"/>
-      <c r="M27" s="4" t="n"/>
-      <c r="N27" s="4" t="n"/>
-      <c r="O27" s="4" t="n"/>
-      <c r="P27" s="4" t="n"/>
-      <c r="Q27" s="4" t="inlineStr">
+      <c r="I28" s="4" t="n"/>
+      <c r="J28" s="4" t="n"/>
+      <c r="K28" s="4" t="n"/>
+      <c r="L28" s="4" t="n"/>
+      <c r="M28" s="4" t="n"/>
+      <c r="N28" s="4" t="n"/>
+      <c r="O28" s="4" t="n"/>
+      <c r="P28" s="4" t="n"/>
+      <c r="Q28" s="4" t="inlineStr">
         <is>
           <t>NKA; RW</t>
         </is>
       </c>
-      <c r="R27" s="4" t="n"/>
-      <c r="S27" s="4" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>BFO:0000015</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>process</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>occurrent</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>An occurrent that has temporal proper parts and for some time t.</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
+      <c r="R28" s="4" t="n"/>
+      <c r="S28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>BCIO:043000</t>
+          <t>BFO:0000015</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>process attribute</t>
+          <t>process</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>process profile</t>
+          <t>occurrent</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>A process profile that is an attribute of a process.</t>
+          <t>An occurrent that has temporal proper parts and for some time t.</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1791,70 +1801,97 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>BCIO:043000</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>process attribute</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>process profile</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>A process profile that is an attribute of a process.</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>BFO:0000144</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>process profile</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>b is a process_profile =Def. there is some process c such that b process_profile_of c (axiom label in BFO2 Reference: [093-002])</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="n"/>
-      <c r="B31" s="2" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="2" t="n"/>
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>subjective severity of potentially traumatic experience</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>potentially traumatic experience severity</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>&lt;Potentially traumatic experience severity&gt; that is subjectively experienced by a person.</t>
         </is>
       </c>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="2" t="n"/>
-      <c r="G31" s="2" t="n"/>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>Pre-proposed</t>
         </is>
       </c>
-      <c r="I31" s="2" t="n"/>
-      <c r="J31" s="2" t="n"/>
-      <c r="K31" s="2" t="n"/>
-      <c r="L31" s="2" t="n"/>
-      <c r="M31" s="2" t="inlineStr">
+      <c r="I32" s="2" t="n"/>
+      <c r="J32" s="2" t="n"/>
+      <c r="K32" s="2" t="n"/>
+      <c r="L32" s="2" t="n"/>
+      <c r="M32" s="2" t="inlineStr">
         <is>
           <t>dimension</t>
         </is>
       </c>
-      <c r="N31" s="2" t="n"/>
-      <c r="O31" s="2" t="n"/>
-      <c r="P31" s="2" t="n"/>
-      <c r="Q31" s="2" t="n"/>
-      <c r="R31" s="2" t="n"/>
-      <c r="S31" s="2" t="n"/>
+      <c r="N32" s="2" t="n"/>
+      <c r="O32" s="2" t="n"/>
+      <c r="P32" s="2" t="n"/>
+      <c r="Q32" s="2" t="n"/>
+      <c r="R32" s="2" t="n"/>
+      <c r="S32" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update experience of interpersonal abuse in TSO classes.xlsx
</commit_message>
<xml_diff>
--- a/TSO classes.xlsx
+++ b/TSO classes.xlsx
@@ -790,7 +790,7 @@
           <t>An &lt;experience of interpersonal abuse&gt; that occurs in a familial or caretaking relationship.</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="n"/>
       <c r="F7" s="3" t="inlineStr">
         <is>
           <t>includes sub-classes: child physical abuse, child sexual abuse, intimate partner violence, elder abuse</t>
@@ -917,41 +917,45 @@
       <c r="S9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n"/>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>TSTO:0000026</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>experience of interpersonal abuse</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>A &lt;potentially traumatic experience&gt; that involves repeated abuse by one or more other people.</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="n"/>
-      <c r="J10" s="2" t="n"/>
-      <c r="K10" s="2" t="n"/>
-      <c r="L10" s="2" t="n"/>
-      <c r="M10" s="2" t="n"/>
-      <c r="N10" s="2" t="n"/>
-      <c r="O10" s="2" t="n"/>
-      <c r="P10" s="2" t="n"/>
-      <c r="Q10" s="2" t="n"/>
-      <c r="R10" s="2" t="n"/>
-      <c r="S10" s="2" t="n"/>
+      <c r="E10" s="3" t="n"/>
+      <c r="F10" s="3" t="n"/>
+      <c r="G10" s="3" t="n"/>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="n"/>
+      <c r="J10" s="3" t="n"/>
+      <c r="K10" s="3" t="n"/>
+      <c r="L10" s="3" t="n"/>
+      <c r="M10" s="3" t="n"/>
+      <c r="N10" s="3" t="n"/>
+      <c r="O10" s="3" t="n"/>
+      <c r="P10" s="3" t="n"/>
+      <c r="Q10" s="3" t="n"/>
+      <c r="R10" s="3" t="n"/>
+      <c r="S10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add potentially traumatic experience - life stage to TSO classes.xlsx
</commit_message>
<xml_diff>
--- a/TSO classes.xlsx
+++ b/TSO classes.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S32"/>
+  <dimension ref="A1:S33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,87 +452,87 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Definition</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Parent</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Definition</t>
-        </is>
-      </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Informal definition</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Logical definition</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>BFO Entity</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Sub-ontology</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Synonyms</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Entity URL</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Curation status</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Curation note</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Comment</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>BFO Entity</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Curation status</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Fuzzy class</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Why fuzzy</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Curator</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Reviewer</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Reviewer query</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Entity URL</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Sub-ontology</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Curation note</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Informal definition</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Fuzzy class</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Logical definition</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Curator</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Reviewer</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Why fuzzy</t>
         </is>
       </c>
     </row>
@@ -549,22 +549,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>A &lt;potentially traumatic experience attribute&gt; that is whether event(s) were physically experienced, witnessed, or communicated to the person.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>potentially traumatic experience attribute</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience attribute&gt; that is whether event(s) were physically experienced, witnessed, or communicated to the person.</t>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The directness of a person's exposure to a potentially traumatic experience ranges from direct physical impact to one's body, to personally witnessing (seeing, hearing) event(s), to learning about event(s) that happened to other persons (loved ones or others). </t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
           <t>dimension</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The directness of a person's exposure to a potentially traumatic experience ranges from direct physical impact to one's body, to personally witnessing (seeing, hearing) event(s), to learning about event(s) that happened to other persons (loved ones or others). </t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -586,34 +586,34 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
+          <t>A &lt;potentially traumatic experience&gt; that involves actual harm or the perception of potential harm, without human intention to cause harm and that impacts on one or a few people.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves actual harm or the perception of potential harm, without human intention to cause harm and that impacts on one or a few people.</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>includes sub-classes for road traffic accident, fall, animal attack, residential fire, sports-related, weapon-related (unintentional), choking, drowning</t>
-        </is>
-      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Something that happens which causes potential or actual unintended harm.  Note that DISASTERS are similar but usually impact more people and often (not always) natural forces.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n"/>
       <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="n"/>
       <c r="J3" s="2" t="n"/>
       <c r="K3" s="2" t="n"/>
-      <c r="L3" s="2" t="n"/>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="M3" s="2" t="n"/>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Something that happens which causes potential or actual unintended harm.  Note that DISASTERS are similar but usually impact more people and often (not always) natural forces.</t>
+          <t>includes sub-classes for road traffic accident, fall, animal attack, residential fire, sports-related, weapon-related (unintentional), choking, drowning</t>
         </is>
       </c>
       <c r="O3" s="2" t="n"/>
@@ -639,32 +639,32 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
+          <t>A &lt;potentially traumatic experience&gt; that involves the death of a loved one.</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves the death of a loved one.</t>
-        </is>
-      </c>
       <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>need to consult with colleages about sub-classes - probably traumatic bereavement and others but concept of loved one seems to involve close attachment and need not involve positive affection</t>
-        </is>
-      </c>
+      <c r="F4" s="3" t="n"/>
       <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
+      <c r="H4" s="3" t="n"/>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
       <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n"/>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
       <c r="M4" s="3" t="n"/>
-      <c r="N4" s="3" t="n"/>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>need to consult with colleages about sub-classes - probably traumatic bereavement and others but concept of loved one seems to involve close attachment and need not involve positive affection</t>
+        </is>
+      </c>
       <c r="O4" s="3" t="n"/>
       <c r="P4" s="3" t="n"/>
       <c r="Q4" s="3" t="inlineStr">
@@ -684,32 +684,32 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
+          <t>A &lt;potentially traumatic experience&gt; that occurs during or in direct consequence of a discrete catastrophic event or series of events — whether of natural or technological origin — that causes or threatens widespread death, serious injury, destruction of property, or severe disruption to community functioning.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that occurs during or in direct consequence of a discrete catastrophic event or series of events — whether of natural or technological origin — that causes or threatens widespread death, serious injury, destruction of property, or severe disruption to community functioning.</t>
-        </is>
-      </c>
       <c r="E5" s="2" t="n"/>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>includes sub-classes for natural disaster, technological disaster, transportation disaster (and each of those has multiple sub-classes)</t>
-        </is>
-      </c>
+      <c r="F5" s="2" t="n"/>
       <c r="G5" s="2" t="n"/>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="n"/>
       <c r="J5" s="2" t="n"/>
       <c r="K5" s="2" t="n"/>
-      <c r="L5" s="2" t="n"/>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="M5" s="2" t="n"/>
-      <c r="N5" s="2" t="n"/>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>includes sub-classes for natural disaster, technological disaster, transportation disaster (and each of those has multiple sub-classes)</t>
+        </is>
+      </c>
       <c r="O5" s="2" t="n"/>
       <c r="P5" s="2" t="n"/>
       <c r="Q5" s="2" t="inlineStr">
@@ -733,32 +733,32 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
+          <t>A &lt;potentially traumatic experience&gt; that involves  displacement from the person's home area because of physical or political danger or by force.</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves  displacement from the person's home area because of physical or political danger or by force.</t>
-        </is>
-      </c>
       <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>might include sub-classes for refugee experiences, forced migration, prolonged displacement, climate-related displacement</t>
-        </is>
-      </c>
+      <c r="F6" s="3" t="n"/>
       <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
+      <c r="H6" s="3" t="n"/>
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
       <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="n"/>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
       <c r="M6" s="3" t="n"/>
-      <c r="N6" s="3" t="n"/>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>might include sub-classes for refugee experiences, forced migration, prolonged displacement, climate-related displacement</t>
+        </is>
+      </c>
       <c r="O6" s="3" t="n"/>
       <c r="P6" s="3" t="n"/>
       <c r="Q6" s="3" t="inlineStr">
@@ -782,32 +782,32 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
+          <t>An &lt;experience of interpersonal abuse&gt; that occurs in a familial or caretaking relationship.</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
           <t>experience of interpersonal abuse</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>An &lt;experience of interpersonal abuse&gt; that occurs in a familial or caretaking relationship.</t>
-        </is>
-      </c>
       <c r="E7" s="3" t="n"/>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>includes sub-classes: child physical abuse, child sexual abuse, intimate partner violence, elder abuse</t>
-        </is>
-      </c>
+      <c r="F7" s="3" t="n"/>
       <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
+      <c r="H7" s="3" t="n"/>
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="n"/>
       <c r="K7" s="3" t="n"/>
-      <c r="L7" s="3" t="n"/>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
       <c r="M7" s="3" t="n"/>
-      <c r="N7" s="3" t="n"/>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>includes sub-classes: child physical abuse, child sexual abuse, intimate partner violence, elder abuse</t>
+        </is>
+      </c>
       <c r="O7" s="3" t="n"/>
       <c r="P7" s="3" t="n"/>
       <c r="Q7" s="3" t="inlineStr">
@@ -831,32 +831,32 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
+          <t>A &lt;potentially traumatic experience&gt; that involves the person being compelled to provide labor through force, threat, deception, or abuse of power, and without the possibility of free and informed refusal</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves the person being compelled to provide labor through force, threat, deception, or abuse of power, and without the possibility of free and informed refusal</t>
-        </is>
-      </c>
       <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>includes sub-classes for slavery, human trafficking</t>
-        </is>
-      </c>
+      <c r="F8" s="2" t="n"/>
       <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="n"/>
       <c r="J8" s="2" t="n"/>
       <c r="K8" s="2" t="n"/>
-      <c r="L8" s="2" t="n"/>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="M8" s="2" t="n"/>
-      <c r="N8" s="2" t="n"/>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>includes sub-classes for slavery, human trafficking</t>
+        </is>
+      </c>
       <c r="O8" s="2" t="n"/>
       <c r="P8" s="2" t="n"/>
       <c r="Q8" s="2" t="inlineStr">
@@ -880,32 +880,32 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
+          <t>A &lt;potentially traumatic experience&gt; that involves  illness, injury or treatment.</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves  illness, injury or treatment.</t>
-        </is>
-      </c>
       <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>includes sub-classes for injury, illness, treatment experiences (and each of these has sub-classes)</t>
-        </is>
-      </c>
+      <c r="F9" s="3" t="n"/>
       <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
+      <c r="H9" s="3" t="n"/>
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
       <c r="K9" s="3" t="n"/>
-      <c r="L9" s="3" t="n"/>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
       <c r="M9" s="3" t="n"/>
-      <c r="N9" s="3" t="n"/>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>includes sub-classes for injury, illness, treatment experiences (and each of these has sub-classes)</t>
+        </is>
+      </c>
       <c r="O9" s="3" t="n"/>
       <c r="P9" s="3" t="n"/>
       <c r="Q9" s="3" t="inlineStr">
@@ -929,26 +929,26 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
+          <t>A &lt;potentially traumatic experience&gt; that involves repeated abuse by one or more other people.</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
           <t>potentially traumatic experience</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves repeated abuse by one or more other people.</t>
         </is>
       </c>
       <c r="E10" s="3" t="n"/>
       <c r="F10" s="3" t="n"/>
       <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
+      <c r="H10" s="3" t="n"/>
       <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="n"/>
       <c r="K10" s="3" t="n"/>
-      <c r="L10" s="3" t="n"/>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
       <c r="M10" s="3" t="n"/>
       <c r="N10" s="3" t="n"/>
       <c r="O10" s="3" t="n"/>
@@ -970,32 +970,32 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
+          <t>A &lt;potentially traumatic experience&gt; that involves violence perpetrated by one or more other persons, outside of the context of organised armed conflict.</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves violence perpetrated by one or more other persons, outside of the context of organised armed conflict.</t>
-        </is>
-      </c>
       <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>includes sub-classes for physical assault, sexual assault, homicide, abduction-kidnapping, hostage taking, torture</t>
-        </is>
-      </c>
+      <c r="F11" s="3" t="n"/>
       <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
+      <c r="H11" s="3" t="n"/>
       <c r="I11" s="3" t="n"/>
       <c r="J11" s="3" t="n"/>
       <c r="K11" s="3" t="n"/>
-      <c r="L11" s="3" t="n"/>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
       <c r="M11" s="3" t="n"/>
-      <c r="N11" s="3" t="n"/>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>includes sub-classes for physical assault, sexual assault, homicide, abduction-kidnapping, hostage taking, torture</t>
+        </is>
+      </c>
       <c r="O11" s="3" t="n"/>
       <c r="P11" s="3" t="n"/>
       <c r="Q11" s="3" t="inlineStr">
@@ -1019,32 +1019,32 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
+          <t>A &lt;potentially traumatic experience&gt; that involves experience of violence directed at a group of people.</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves experience of violence directed at a group of people.</t>
-        </is>
-      </c>
       <c r="E12" s="3" t="n"/>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>includes sub-classes for mass injury or homicide, terrorism, genocide</t>
-        </is>
-      </c>
+      <c r="F12" s="3" t="n"/>
       <c r="G12" s="3" t="n"/>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
+      <c r="H12" s="3" t="n"/>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
       <c r="K12" s="3" t="n"/>
-      <c r="L12" s="3" t="n"/>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
       <c r="M12" s="3" t="n"/>
-      <c r="N12" s="3" t="n"/>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>includes sub-classes for mass injury or homicide, terrorism, genocide</t>
+        </is>
+      </c>
       <c r="O12" s="3" t="n"/>
       <c r="P12" s="3" t="n"/>
       <c r="Q12" s="3" t="inlineStr">
@@ -1068,32 +1068,32 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
+          <t>A &lt;potentially traumatic experience&gt; that occurs during or in direct consequence of organised armed conflict.</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that occurs during or in direct consequence of organised armed conflict.</t>
-        </is>
-      </c>
       <c r="E13" s="3" t="n"/>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>includes sub-classes for civilian exposure to warfare or armed conflict, combat exposure as a member of armed forces, deployment as a member of armed forces</t>
-        </is>
-      </c>
+      <c r="F13" s="3" t="n"/>
       <c r="G13" s="3" t="n"/>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
+      <c r="H13" s="3" t="n"/>
       <c r="I13" s="3" t="n"/>
       <c r="J13" s="3" t="n"/>
       <c r="K13" s="3" t="n"/>
-      <c r="L13" s="3" t="n"/>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
       <c r="M13" s="3" t="n"/>
-      <c r="N13" s="3" t="n"/>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>includes sub-classes for civilian exposure to warfare or armed conflict, combat exposure as a member of armed forces, deployment as a member of armed forces</t>
+        </is>
+      </c>
       <c r="O13" s="3" t="n"/>
       <c r="P13" s="3" t="n"/>
       <c r="Q13" s="3" t="inlineStr">
@@ -1117,32 +1117,32 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
+          <t>A &lt;potentially traumatic experience&gt; that involves adversity or harm related to the person's perceived race or ethnicity or their racial or ethnic identity.</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves adversity or harm related to the person's perceived race or ethnicity or their racial or ethnic identity.</t>
-        </is>
-      </c>
       <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>includes sub-classes for experiences of racism, hate crimes, micro-agressions, generational trauma</t>
-        </is>
-      </c>
+      <c r="F14" s="3" t="n"/>
       <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
+      <c r="H14" s="3" t="n"/>
       <c r="I14" s="3" t="n"/>
       <c r="J14" s="3" t="n"/>
       <c r="K14" s="3" t="n"/>
-      <c r="L14" s="3" t="n"/>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
       <c r="M14" s="3" t="n"/>
-      <c r="N14" s="3" t="n"/>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>includes sub-classes for experiences of racism, hate crimes, micro-agressions, generational trauma</t>
+        </is>
+      </c>
       <c r="O14" s="3" t="n"/>
       <c r="P14" s="3" t="n"/>
       <c r="Q14" s="3" t="inlineStr">
@@ -1166,32 +1166,32 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
+          <t>A &lt;potentially traumatic experience&gt; that involves being confined by a state or state-sanctioned authority.</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves being confined by a state or state-sanctioned authority.</t>
-        </is>
-      </c>
       <c r="E15" s="3" t="n"/>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">includes sub-classes for incarceration related to crime, concentration camp imprisonment, political imprisonment, war imprisonment </t>
-        </is>
-      </c>
+      <c r="F15" s="3" t="n"/>
       <c r="G15" s="3" t="n"/>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
+      <c r="H15" s="3" t="n"/>
       <c r="I15" s="3" t="n"/>
       <c r="J15" s="3" t="n"/>
       <c r="K15" s="3" t="n"/>
-      <c r="L15" s="3" t="n"/>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
       <c r="M15" s="3" t="n"/>
-      <c r="N15" s="3" t="n"/>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">includes sub-classes for incarceration related to crime, concentration camp imprisonment, political imprisonment, war imprisonment </t>
+        </is>
+      </c>
       <c r="O15" s="3" t="n"/>
       <c r="P15" s="3" t="n"/>
       <c r="Q15" s="3" t="inlineStr">
@@ -1215,32 +1215,32 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
+          <t>A &lt;potentially traumatic experience&gt; that involves ongoing exposure to a social environment in which violence is common.</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves ongoing exposure to a social environment in which violence is common.</t>
-        </is>
-      </c>
       <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">includes sub-classes for community evironment of violence; school enviroment of violence; workplace enviroment of violence; environment of violence related to gender, ethnicity or other marginalized identity  </t>
-        </is>
-      </c>
+      <c r="F16" s="3" t="n"/>
       <c r="G16" s="3" t="n"/>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
+      <c r="H16" s="3" t="n"/>
       <c r="I16" s="3" t="n"/>
       <c r="J16" s="3" t="n"/>
       <c r="K16" s="3" t="n"/>
-      <c r="L16" s="3" t="n"/>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
       <c r="M16" s="3" t="n"/>
-      <c r="N16" s="3" t="n"/>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">includes sub-classes for community evironment of violence; school enviroment of violence; workplace enviroment of violence; environment of violence related to gender, ethnicity or other marginalized identity  </t>
+        </is>
+      </c>
       <c r="O16" s="3" t="n"/>
       <c r="P16" s="3" t="n"/>
       <c r="Q16" s="3" t="inlineStr">
@@ -1264,15 +1264,15 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>A process that is the sum of the totality of processes taking place in the spatiotemporal region occupied by a material entity or site, including processes on the surface of the entity or within the cavities to which it serves as host</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
           <t>process</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>A process that is the sum of the totality of processes taking place in the spatiotemporal region occupied by a material entity or site, including processes on the surface of the entity or within the cavities to which it serves as host</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -1291,26 +1291,26 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
+          <t>A personal attribute that is the kinship connection of the person a person who has has a specified potentially traumatic experience.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
           <t>personal attribute</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>A personal attribute that is the kinship connection of the person a person who has has a specified potentially traumatic experience.</t>
         </is>
       </c>
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="n"/>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="H18" s="2" t="n"/>
       <c r="I18" s="2" t="n"/>
       <c r="J18" s="2" t="n"/>
       <c r="K18" s="2" t="n"/>
-      <c r="L18" s="2" t="n"/>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="M18" s="2" t="n"/>
       <c r="N18" s="2" t="n"/>
       <c r="O18" s="2" t="n"/>
@@ -1332,26 +1332,26 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
+          <t>The aspect of &lt;potentially traumatic experience severity&gt; that is an objective degree of intensity, damage, or risk</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
           <t>potentially traumatic experience severity</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>The aspect of &lt;potentially traumatic experience severity&gt; that is an objective degree of intensity, damage, or risk</t>
         </is>
       </c>
       <c r="E19" s="2" t="n"/>
       <c r="F19" s="2" t="n"/>
       <c r="G19" s="2" t="n"/>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
+      <c r="H19" s="2" t="n"/>
       <c r="I19" s="2" t="n"/>
       <c r="J19" s="2" t="n"/>
       <c r="K19" s="2" t="n"/>
-      <c r="L19" s="2" t="n"/>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
           <t>dimension</t>
@@ -1377,15 +1377,15 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
+          <t>An entity that unfolds itself in time or it is the instantaneous boundary of such an entity</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
           <t>entity</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>An entity that unfolds itself in time or it is the instantaneous boundary of such an entity</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -1404,15 +1404,15 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
+          <t>A history that is of a person.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
           <t>history</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>A history that is of a person.</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -1431,15 +1431,15 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
+          <t>A process that is part of a personal history.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
           <t>process</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>A process that is part of a personal history.</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -1458,20 +1458,20 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
+          <t>A &lt;personal history part&gt; that may lead to some traumatic stress response.</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;personal history part&gt; that may lead to some traumatic stress response.</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>The use of 'may lead to' is to be interpreted as in at least one case having done so. The focus on 'experience' is designed to recognise that there are other semantic hierarchies for events such as disasters, accidents etc. and that this hierarchy is aimed at classifying the experience of these not the events themselves.</t>
-        </is>
-      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Something that a person has experienced that may lead in some cases to some kind of traumatic stress response.</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="n"/>
       <c r="G23" s="3" t="inlineStr">
         <is>
           <t>process</t>
@@ -1479,7 +1479,7 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>PTEO</t>
         </is>
       </c>
       <c r="I23" s="3" t="n"/>
@@ -1487,13 +1487,13 @@
       <c r="K23" s="3" t="n"/>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>PTEO</t>
+          <t>Proposed</t>
         </is>
       </c>
       <c r="M23" s="3" t="n"/>
       <c r="N23" s="3" t="inlineStr">
         <is>
-          <t>Something that a person has experienced that may lead in some cases to some kind of traumatic stress response.</t>
+          <t>The use of 'may lead to' is to be interpreted as in at least one case having done so. The focus on 'experience' is designed to recognise that there are other semantic hierarchies for events such as disasters, accidents etc. and that this hierarchy is aimed at classifying the experience of these not the events themselves.</t>
         </is>
       </c>
       <c r="O23" s="3" t="n"/>
@@ -1519,40 +1519,40 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
+          <t>A &lt;potentially traumatic experience attribute&gt; that is the degree of human agency involved in causing the event(s) experienced</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
           <t>potentially traumatic experience attribute</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience attribute&gt; that is the degree of human agency involved in causing the event(s) experienced</t>
-        </is>
-      </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>intentionality</t>
+          <t>The degree to which the causal process involved in the the event(s) which are/were experienced involved human agency / intention to harm.</t>
         </is>
       </c>
       <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="n"/>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>intentionality</t>
+        </is>
+      </c>
       <c r="J24" s="2" t="n"/>
       <c r="K24" s="2" t="n"/>
-      <c r="L24" s="2" t="n"/>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
           <t>dimension</t>
         </is>
       </c>
-      <c r="N24" s="2" t="inlineStr">
-        <is>
-          <t>The degree to which the causal process involved in the the event(s) which are/were experienced involved human agency / intention to harm.</t>
-        </is>
-      </c>
+      <c r="N24" s="2" t="n"/>
       <c r="O24" s="2" t="n"/>
       <c r="P24" s="2" t="n"/>
       <c r="Q24" s="2" t="inlineStr">
@@ -1564,158 +1564,146 @@
       <c r="S24" s="2" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr"/>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>potentially traumatic experience - life stage</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A &lt;potentially traumatic experience attribute&gt; that is the life stage in which the event or events were experienced by a person </t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>potentially traumatic experience attribute</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr"/>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>PTEs may be experienced in one or more life stages</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr"/>
+      <c r="P25" s="2" t="inlineStr"/>
+      <c r="Q25" s="2" t="inlineStr"/>
+      <c r="R25" s="2" t="inlineStr"/>
+      <c r="S25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>TSTO:0000021</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>potentially traumatic experience attribute</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A characteristic of a potentially traumatic experience </t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>process attribute</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A characteristic of a potentially traumatic experience </t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
-      <c r="G25" s="3" t="n"/>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Attributes of PTEs include their time course, severity, degree of human agency involved in the event, nature of exposure (direct vs indirect)</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="n"/>
+      <c r="G26" s="3" t="n"/>
+      <c r="H26" s="3" t="n"/>
+      <c r="I26" s="3" t="n"/>
+      <c r="J26" s="3" t="n"/>
+      <c r="K26" s="3" t="n"/>
+      <c r="L26" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="I25" s="3" t="n"/>
-      <c r="J25" s="3" t="n"/>
-      <c r="K25" s="3" t="n"/>
-      <c r="L25" s="3" t="n"/>
-      <c r="M25" s="3" t="n"/>
-      <c r="N25" s="3" t="inlineStr">
-        <is>
-          <t>Attributes of PTEs include their time course, severity, degree of human agency involved in the event, nature of exposure (direct vs indirect)</t>
-        </is>
-      </c>
-      <c r="O25" s="3" t="n"/>
-      <c r="P25" s="3" t="n"/>
-      <c r="Q25" s="3" t="inlineStr">
+      <c r="M26" s="3" t="n"/>
+      <c r="N26" s="3" t="n"/>
+      <c r="O26" s="3" t="n"/>
+      <c r="P26" s="3" t="n"/>
+      <c r="Q26" s="3" t="inlineStr">
         <is>
           <t>NKA</t>
         </is>
       </c>
-      <c r="R25" s="3" t="n"/>
-      <c r="S25" s="3" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>TSTO:0000018</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience severity</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience attribute</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience attribute&gt; that is the severity of the event(s) experienced.</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>intensity</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>Severity might be seen as a combination of several other attributes listed here - but I think we often think of this as an independent dimension.  Should there be sub-classes for obective severity and subjective or perceived severity, or for objective and perceived life threat?   - to be discussed with colleagues</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="n"/>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="n"/>
-      <c r="J26" s="2" t="n"/>
-      <c r="K26" s="2" t="n"/>
-      <c r="L26" s="2" t="n"/>
-      <c r="M26" s="2" t="inlineStr">
-        <is>
-          <t>dimension</t>
-        </is>
-      </c>
-      <c r="N26" s="2" t="inlineStr">
-        <is>
-          <t>The severity of a PTE relates to its degree of intensity, damage, or risk and includes both objective event factors and the subjective experience of the person.</t>
-        </is>
-      </c>
-      <c r="O26" s="2" t="n"/>
-      <c r="P26" s="2" t="n"/>
-      <c r="Q26" s="2" t="inlineStr">
-        <is>
-          <t>NKA</t>
-        </is>
-      </c>
-      <c r="R26" s="2" t="n"/>
-      <c r="S26" s="2" t="n"/>
+      <c r="R26" s="3" t="n"/>
+      <c r="S26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>TSTO:0000019</t>
+          <t>TSTO:0000018</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>potentially traumatic experience time course</t>
+          <t>potentially traumatic experience severity</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
+          <t>A &lt;potentially traumatic experience attribute&gt; that is the severity of the event(s) experienced.</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
           <t>potentially traumatic experience attribute</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience attribute&gt; that is the chronicity, duration, and frequency of the event(s) experienced.</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>include sub-classes for chronicity, frequency, duration, age at onset</t>
-        </is>
-      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>The severity of a PTE relates to its degree of intensity, damage, or risk and includes both objective event factors and the subjective experience of the person.</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="n"/>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
-      <c r="I27" s="2" t="n"/>
+      <c r="H27" s="2" t="n"/>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>intensity</t>
+        </is>
+      </c>
       <c r="J27" s="2" t="n"/>
       <c r="K27" s="2" t="n"/>
-      <c r="L27" s="2" t="n"/>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
           <t>dimension</t>
         </is>
       </c>
-      <c r="N27" s="2" t="n"/>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>Severity might be seen as a combination of several other attributes listed here - but I think we often think of this as an independent dimension.  Should there be sub-classes for obective severity and subjective or perceived severity, or for objective and perceived life threat?   - to be discussed with colleagues</t>
+        </is>
+      </c>
       <c r="O27" s="2" t="n"/>
       <c r="P27" s="2" t="n"/>
       <c r="Q27" s="2" t="inlineStr">
@@ -1727,103 +1715,129 @@
       <c r="S27" s="2" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>TSTO:0000019</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>potentially traumatic experience time course</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;potentially traumatic experience attribute&gt; that is the chronicity, duration, and frequency of the event(s) experienced.</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>potentially traumatic experience attribute</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="n"/>
+      <c r="I28" s="2" t="n"/>
+      <c r="J28" s="2" t="n"/>
+      <c r="K28" s="2" t="n"/>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>dimension</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>include sub-classes for chronicity, frequency, duration, age at onset</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="n"/>
+      <c r="P28" s="2" t="n"/>
+      <c r="Q28" s="2" t="inlineStr">
+        <is>
+          <t>NKA</t>
+        </is>
+      </c>
+      <c r="R28" s="2" t="n"/>
+      <c r="S28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>TSTO:0000020</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>potentially traumatic experience type</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>An attribute of a potentially traumatic experience that is the type of event(s) experienced by a person.</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>potentially traumatic experience attribute</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>An attribute of a potentially traumatic experience that is the type of event(s) experienced by a person.</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E29" s="4" t="n"/>
+      <c r="F29" s="4" t="n"/>
+      <c r="G29" s="4" t="n"/>
+      <c r="H29" s="4" t="n"/>
+      <c r="I29" s="4" t="inlineStr">
         <is>
           <t>event type</t>
         </is>
       </c>
-      <c r="F28" s="4" t="n"/>
-      <c r="G28" s="4" t="n"/>
-      <c r="H28" s="4" t="inlineStr">
+      <c r="J29" s="4" t="n"/>
+      <c r="K29" s="4" t="n"/>
+      <c r="L29" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="I28" s="4" t="n"/>
-      <c r="J28" s="4" t="n"/>
-      <c r="K28" s="4" t="n"/>
-      <c r="L28" s="4" t="n"/>
-      <c r="M28" s="4" t="n"/>
-      <c r="N28" s="4" t="n"/>
-      <c r="O28" s="4" t="n"/>
-      <c r="P28" s="4" t="n"/>
-      <c r="Q28" s="4" t="inlineStr">
+      <c r="M29" s="4" t="n"/>
+      <c r="N29" s="4" t="n"/>
+      <c r="O29" s="4" t="n"/>
+      <c r="P29" s="4" t="n"/>
+      <c r="Q29" s="4" t="inlineStr">
         <is>
           <t>NKA; RW</t>
         </is>
       </c>
-      <c r="R28" s="4" t="n"/>
-      <c r="S28" s="4" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>BFO:0000015</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>process</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>occurrent</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>An occurrent that has temporal proper parts and for some time t.</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
+      <c r="R29" s="4" t="n"/>
+      <c r="S29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>BCIO:043000</t>
+          <t>BFO:0000015</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>process attribute</t>
+          <t>process</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>process profile</t>
+          <t>An occurrent that has temporal proper parts and for some time t.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>A process profile that is an attribute of a process.</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
+          <t>occurrent</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -1832,70 +1846,97 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>BCIO:043000</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>process attribute</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>A process profile that is an attribute of a process.</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>process profile</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>BFO:0000144</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>process profile</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>b is a process_profile =Def. there is some process c such that b process_profile_of c (axiom label in BFO2 Reference: [093-002])</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>b is a process_profile =Def. there is some process c such that b process_profile_of c (axiom label in BFO2 Reference: [093-002])</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="2" t="n"/>
-      <c r="B32" s="2" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="2" t="n"/>
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>subjective severity of potentially traumatic experience</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>&lt;Potentially traumatic experience severity&gt; that is subjectively experienced by a person.</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>potentially traumatic experience severity</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>&lt;Potentially traumatic experience severity&gt; that is subjectively experienced by a person.</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="n"/>
-      <c r="F32" s="2" t="n"/>
-      <c r="G32" s="2" t="n"/>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2" t="n"/>
+      <c r="H33" s="2" t="n"/>
+      <c r="I33" s="2" t="n"/>
+      <c r="J33" s="2" t="n"/>
+      <c r="K33" s="2" t="n"/>
+      <c r="L33" s="2" t="inlineStr">
         <is>
           <t>Pre-proposed</t>
         </is>
       </c>
-      <c r="I32" s="2" t="n"/>
-      <c r="J32" s="2" t="n"/>
-      <c r="K32" s="2" t="n"/>
-      <c r="L32" s="2" t="n"/>
-      <c r="M32" s="2" t="inlineStr">
+      <c r="M33" s="2" t="inlineStr">
         <is>
           <t>dimension</t>
         </is>
       </c>
-      <c r="N32" s="2" t="n"/>
-      <c r="O32" s="2" t="n"/>
-      <c r="P32" s="2" t="n"/>
-      <c r="Q32" s="2" t="n"/>
-      <c r="R32" s="2" t="n"/>
-      <c r="S32" s="2" t="n"/>
+      <c r="N33" s="2" t="n"/>
+      <c r="O33" s="2" t="n"/>
+      <c r="P33" s="2" t="n"/>
+      <c r="Q33" s="2" t="n"/>
+      <c r="R33" s="2" t="n"/>
+      <c r="S33" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update potentially traumatic experience attribute in TSO classes.xlsx
</commit_message>
<xml_diff>
--- a/TSO classes.xlsx
+++ b/TSO classes.xlsx
@@ -1564,7 +1564,7 @@
       <c r="S24" s="2" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr"/>
+      <c r="A25" s="2" t="n"/>
       <c r="B25" s="2" t="inlineStr">
         <is>
           <t>potentially traumatic experience - life stage</t>
@@ -1580,29 +1580,29 @@
           <t>potentially traumatic experience attribute</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="2" t="inlineStr"/>
-      <c r="G25" s="2" t="inlineStr"/>
-      <c r="H25" s="2" t="inlineStr"/>
-      <c r="I25" s="2" t="inlineStr"/>
-      <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="inlineStr"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n"/>
+      <c r="I25" s="2" t="n"/>
+      <c r="J25" s="2" t="n"/>
+      <c r="K25" s="2" t="n"/>
       <c r="L25" s="2" t="inlineStr">
         <is>
           <t>Pre-proposed</t>
         </is>
       </c>
-      <c r="M25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="n"/>
       <c r="N25" s="2" t="inlineStr">
         <is>
           <t>PTEs may be experienced in one or more life stages</t>
         </is>
       </c>
-      <c r="O25" s="2" t="inlineStr"/>
-      <c r="P25" s="2" t="inlineStr"/>
-      <c r="Q25" s="2" t="inlineStr"/>
-      <c r="R25" s="2" t="inlineStr"/>
-      <c r="S25" s="2" t="inlineStr"/>
+      <c r="O25" s="2" t="n"/>
+      <c r="P25" s="2" t="n"/>
+      <c r="Q25" s="2" t="n"/>
+      <c r="R25" s="2" t="n"/>
+      <c r="S25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A characteristic of a potentially traumatic experience </t>
+          <t xml:space="preserve">A &lt;process attribute" that is a characteristic of a potentially traumatic experience </t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add experience of non-familial interpersonal abuse to TSO classes.xlsx
</commit_message>
<xml_diff>
--- a/TSO classes.xlsx
+++ b/TSO classes.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S33"/>
+  <dimension ref="A1:S34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1105,68 +1105,64 @@
       <c r="S13" s="3" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>TSTO:0000011</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>experience of racial trauma</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves adversity or harm related to the person's perceived race or ethnicity or their racial or ethnic identity.</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
-      <c r="J14" s="3" t="n"/>
-      <c r="K14" s="3" t="n"/>
-      <c r="L14" s="3" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="M14" s="3" t="n"/>
-      <c r="N14" s="3" t="inlineStr">
-        <is>
-          <t>includes sub-classes for experiences of racism, hate crimes, micro-agressions, generational trauma</t>
-        </is>
-      </c>
-      <c r="O14" s="3" t="n"/>
-      <c r="P14" s="3" t="n"/>
-      <c r="Q14" s="3" t="inlineStr">
-        <is>
-          <t>NKA</t>
-        </is>
-      </c>
-      <c r="R14" s="3" t="n"/>
-      <c r="S14" s="3" t="n"/>
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>experience of non-familial interpersonal abuse</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>An &lt;experience of interpersonal abuse&gt; that occurs in a non-familial relationship.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>experience of interpersonal abuse</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Non-familial interpersonal abuse includes bullying or harassment by other persons known or unknown to the person.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">includes sub-classes for bullying and various forms of harassment.  Distinguish from interpersonal physical violence, with which it may co-occur. </t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr"/>
+      <c r="P14" s="2" t="inlineStr"/>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>TSTO:0000006</t>
+          <t>TSTO:0000011</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>experience of state-sanctioned incarceration</t>
+          <t>experience of racial trauma</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves being confined by a state or state-sanctioned authority.</t>
+          <t>A &lt;potentially traumatic experience&gt; that involves adversity or harm related to the person's perceived race or ethnicity or their racial or ethnic identity.</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1189,7 +1185,7 @@
       <c r="M15" s="3" t="n"/>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">includes sub-classes for incarceration related to crime, concentration camp imprisonment, political imprisonment, war imprisonment </t>
+          <t>includes sub-classes for experiences of racism, hate crimes, micro-agressions, generational trauma</t>
         </is>
       </c>
       <c r="O15" s="3" t="n"/>
@@ -1205,17 +1201,17 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>TSTO:0000012</t>
+          <t>TSTO:0000006</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>experience of violent social environment</t>
+          <t>experience of state-sanctioned incarceration</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience&gt; that involves ongoing exposure to a social environment in which violence is common.</t>
+          <t>A &lt;potentially traumatic experience&gt; that involves being confined by a state or state-sanctioned authority.</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -1238,7 +1234,7 @@
       <c r="M16" s="3" t="n"/>
       <c r="N16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">includes sub-classes for community evironment of violence; school enviroment of violence; workplace enviroment of violence; environment of violence related to gender, ethnicity or other marginalized identity  </t>
+          <t xml:space="preserve">includes sub-classes for incarceration related to crime, concentration camp imprisonment, political imprisonment, war imprisonment </t>
         </is>
       </c>
       <c r="O16" s="3" t="n"/>
@@ -1252,92 +1248,100 @@
       <c r="S16" s="3" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>TSTO:0000012</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>experience of violent social environment</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;potentially traumatic experience&gt; that involves ongoing exposure to a social environment in which violence is common.</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>potentially traumatic experience</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" s="3" t="n"/>
+      <c r="G17" s="3" t="n"/>
+      <c r="H17" s="3" t="n"/>
+      <c r="I17" s="3" t="n"/>
+      <c r="J17" s="3" t="n"/>
+      <c r="K17" s="3" t="n"/>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="n"/>
+      <c r="N17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">includes sub-classes for community evironment of violence; school enviroment of violence; workplace enviroment of violence; environment of violence related to gender, ethnicity or other marginalized identity  </t>
+        </is>
+      </c>
+      <c r="O17" s="3" t="n"/>
+      <c r="P17" s="3" t="n"/>
+      <c r="Q17" s="3" t="inlineStr">
+        <is>
+          <t>NKA</t>
+        </is>
+      </c>
+      <c r="R17" s="3" t="n"/>
+      <c r="S17" s="3" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>BFO:0000182</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>history</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>A process that is the sum of the totality of processes taking place in the spatiotemporal region occupied by a material entity or site, including processes on the surface of the entity or within the cavities to which it serves as host</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>TSTO:0000022</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>kinship relationship with potentially traumatic experience target</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>A personal attribute that is the kinship connection of the person a person who has has a specified potentially traumatic experience.</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="n"/>
-      <c r="G18" s="2" t="n"/>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="n"/>
-      <c r="J18" s="2" t="n"/>
-      <c r="K18" s="2" t="n"/>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="n"/>
-      <c r="N18" s="2" t="n"/>
-      <c r="O18" s="2" t="n"/>
-      <c r="P18" s="2" t="n"/>
-      <c r="Q18" s="2" t="n"/>
-      <c r="R18" s="2" t="n"/>
-      <c r="S18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>TSTO:0000023</t>
+          <t>TSTO:0000022</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>objective severity of potentially traumatic event(s)</t>
+          <t>kinship relationship with potentially traumatic experience target</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>The aspect of &lt;potentially traumatic experience severity&gt; that is an objective degree of intensity, damage, or risk</t>
+          <t>A personal attribute that is the kinship connection of the person a person who has has a specified potentially traumatic experience.</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>potentially traumatic experience severity</t>
+          <t>personal attribute</t>
         </is>
       </c>
       <c r="E19" s="2" t="n"/>
@@ -1352,11 +1356,7 @@
           <t>Pre-proposed</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr">
-        <is>
-          <t>dimension</t>
-        </is>
-      </c>
+      <c r="M19" s="2" t="n"/>
       <c r="N19" s="2" t="n"/>
       <c r="O19" s="2" t="n"/>
       <c r="P19" s="2" t="n"/>
@@ -1365,51 +1365,69 @@
       <c r="S19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>BFO:0000003</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>occurrent</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>An entity that unfolds itself in time or it is the instantaneous boundary of such an entity</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>entity</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>TSTO:0000023</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>objective severity of potentially traumatic event(s)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>The aspect of &lt;potentially traumatic experience severity&gt; that is an objective degree of intensity, damage, or risk</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>potentially traumatic experience severity</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="2" t="n"/>
+      <c r="J20" s="2" t="n"/>
+      <c r="K20" s="2" t="n"/>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>dimension</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="n"/>
+      <c r="O20" s="2" t="n"/>
+      <c r="P20" s="2" t="n"/>
+      <c r="Q20" s="2" t="n"/>
+      <c r="R20" s="2" t="n"/>
+      <c r="S20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BCIO:015161</t>
+          <t>BFO:0000003</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>personal history</t>
+          <t>occurrent</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>A history that is of a person.</t>
+          <t>An entity that unfolds itself in time or it is the instantaneous boundary of such an entity</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>history</t>
+          <t>entity</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -1421,170 +1439,152 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>BCIO:015161</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>personal history</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>A history that is of a person.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>history</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>BCIO:050487</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>A process that is part of a personal history.</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>TSTO:0000001</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>potentially traumatic experience</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>A &lt;personal history part&gt; that may lead to some traumatic stress response.</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>Something that a person has experienced that may lead in some cases to some kind of traumatic stress response.</t>
         </is>
       </c>
-      <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="F24" s="3" t="n"/>
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr">
+      <c r="H24" s="3" t="inlineStr">
         <is>
           <t>PTEO</t>
         </is>
       </c>
-      <c r="I23" s="3" t="n"/>
-      <c r="J23" s="3" t="n"/>
-      <c r="K23" s="3" t="n"/>
-      <c r="L23" s="3" t="inlineStr">
+      <c r="I24" s="3" t="n"/>
+      <c r="J24" s="3" t="n"/>
+      <c r="K24" s="3" t="n"/>
+      <c r="L24" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="M23" s="3" t="n"/>
-      <c r="N23" s="3" t="inlineStr">
+      <c r="M24" s="3" t="n"/>
+      <c r="N24" s="3" t="inlineStr">
         <is>
           <t>The use of 'may lead to' is to be interpreted as in at least one case having done so. The focus on 'experience' is designed to recognise that there are other semantic hierarchies for events such as disasters, accidents etc. and that this hierarchy is aimed at classifying the experience of these not the events themselves.</t>
         </is>
       </c>
-      <c r="O23" s="3" t="n"/>
-      <c r="P23" s="3" t="n"/>
-      <c r="Q23" s="3" t="inlineStr">
+      <c r="O24" s="3" t="n"/>
+      <c r="P24" s="3" t="n"/>
+      <c r="Q24" s="3" t="inlineStr">
         <is>
           <t>NKA</t>
         </is>
       </c>
-      <c r="R23" s="3" t="n"/>
-      <c r="S23" s="3" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="R24" s="3" t="n"/>
+      <c r="S24" s="3" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>TSTO:0000016</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">potentially traumatic experience - degree of human agency </t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>A &lt;potentially traumatic experience attribute&gt; that is the degree of human agency involved in causing the event(s) experienced</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>potentially traumatic experience attribute</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>The degree to which the causal process involved in the the event(s) which are/were experienced involved human agency / intention to harm.</t>
         </is>
       </c>
-      <c r="F24" s="2" t="n"/>
-      <c r="G24" s="2" t="n"/>
-      <c r="H24" s="2" t="n"/>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>intentionality</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="n"/>
-      <c r="K24" s="2" t="n"/>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="inlineStr">
-        <is>
-          <t>dimension</t>
-        </is>
-      </c>
-      <c r="N24" s="2" t="n"/>
-      <c r="O24" s="2" t="n"/>
-      <c r="P24" s="2" t="n"/>
-      <c r="Q24" s="2" t="inlineStr">
-        <is>
-          <t>NKA</t>
-        </is>
-      </c>
-      <c r="R24" s="2" t="n"/>
-      <c r="S24" s="2" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="n"/>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience - life stage</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A &lt;potentially traumatic experience attribute&gt; that is the life stage in which the event or events were experienced by a person </t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience attribute</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="n"/>
       <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="n"/>
       <c r="H25" s="2" t="n"/>
-      <c r="I25" s="2" t="n"/>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>intentionality</t>
+        </is>
+      </c>
       <c r="J25" s="2" t="n"/>
       <c r="K25" s="2" t="n"/>
       <c r="L25" s="2" t="inlineStr">
@@ -1592,142 +1592,126 @@
           <t>Pre-proposed</t>
         </is>
       </c>
-      <c r="M25" s="2" t="n"/>
-      <c r="N25" s="2" t="inlineStr">
-        <is>
-          <t>PTEs may be experienced in one or more life stages</t>
-        </is>
-      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>dimension</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="n"/>
       <c r="O25" s="2" t="n"/>
       <c r="P25" s="2" t="n"/>
-      <c r="Q25" s="2" t="n"/>
+      <c r="Q25" s="2" t="inlineStr">
+        <is>
+          <t>NKA</t>
+        </is>
+      </c>
       <c r="R25" s="2" t="n"/>
       <c r="S25" s="2" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="2" t="n"/>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>potentially traumatic experience - life stage</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A &lt;potentially traumatic experience attribute&gt; that is the life stage in which the event or events were experienced by a person </t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>potentially traumatic experience attribute</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
+      <c r="I26" s="2" t="n"/>
+      <c r="J26" s="2" t="n"/>
+      <c r="K26" s="2" t="n"/>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="n"/>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>PTEs may be experienced in one or more life stages</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="n"/>
+      <c r="P26" s="2" t="n"/>
+      <c r="Q26" s="2" t="n"/>
+      <c r="R26" s="2" t="n"/>
+      <c r="S26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>TSTO:0000021</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>potentially traumatic experience attribute</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">A &lt;process attribute&gt; that is a characteristic of a potentially traumatic experience </t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>process attribute</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="E27" s="3" t="inlineStr">
         <is>
           <t>Attributes of PTEs include their time course, severity, degree of human agency involved in the event, nature of exposure (direct vs indirect)</t>
         </is>
       </c>
-      <c r="F26" s="3" t="n"/>
-      <c r="G26" s="3" t="n"/>
-      <c r="H26" s="3" t="n"/>
-      <c r="I26" s="3" t="n"/>
-      <c r="J26" s="3" t="n"/>
-      <c r="K26" s="3" t="n"/>
-      <c r="L26" s="3" t="inlineStr">
+      <c r="F27" s="3" t="n"/>
+      <c r="G27" s="3" t="n"/>
+      <c r="H27" s="3" t="n"/>
+      <c r="I27" s="3" t="n"/>
+      <c r="J27" s="3" t="n"/>
+      <c r="K27" s="3" t="n"/>
+      <c r="L27" s="3" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="M26" s="3" t="n"/>
-      <c r="N26" s="3" t="n"/>
-      <c r="O26" s="3" t="n"/>
-      <c r="P26" s="3" t="n"/>
-      <c r="Q26" s="3" t="inlineStr">
+      <c r="M27" s="3" t="n"/>
+      <c r="N27" s="3" t="n"/>
+      <c r="O27" s="3" t="n"/>
+      <c r="P27" s="3" t="n"/>
+      <c r="Q27" s="3" t="inlineStr">
         <is>
           <t>NKA</t>
         </is>
       </c>
-      <c r="R26" s="3" t="n"/>
-      <c r="S26" s="3" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>TSTO:0000018</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience severity</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>A &lt;potentially traumatic experience attribute&gt; that is the severity of the event(s) experienced.</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>potentially traumatic experience attribute</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>The severity of a PTE relates to its degree of intensity, damage, or risk and includes both objective event factors and the subjective experience of the person.</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="n"/>
-      <c r="G27" s="2" t="n"/>
-      <c r="H27" s="2" t="n"/>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>intensity</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="n"/>
-      <c r="K27" s="2" t="n"/>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
-      <c r="M27" s="2" t="inlineStr">
-        <is>
-          <t>dimension</t>
-        </is>
-      </c>
-      <c r="N27" s="2" t="inlineStr">
-        <is>
-          <t>Severity might be seen as a combination of several other attributes listed here - but I think we often think of this as an independent dimension.  Should there be sub-classes for obective severity and subjective or perceived severity, or for objective and perceived life threat?   - to be discussed with colleagues</t>
-        </is>
-      </c>
-      <c r="O27" s="2" t="n"/>
-      <c r="P27" s="2" t="n"/>
-      <c r="Q27" s="2" t="inlineStr">
-        <is>
-          <t>NKA</t>
-        </is>
-      </c>
-      <c r="R27" s="2" t="n"/>
-      <c r="S27" s="2" t="n"/>
+      <c r="R27" s="3" t="n"/>
+      <c r="S27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>TSTO:0000019</t>
+          <t>TSTO:0000018</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>potentially traumatic experience time course</t>
+          <t>potentially traumatic experience severity</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>A &lt;potentially traumatic experience attribute&gt; that is the chronicity, duration, and frequency of the event(s) experienced.</t>
+          <t>A &lt;potentially traumatic experience attribute&gt; that is the severity of the event(s) experienced.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1735,11 +1719,19 @@
           <t>potentially traumatic experience attribute</t>
         </is>
       </c>
-      <c r="E28" s="2" t="n"/>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>The severity of a PTE relates to its degree of intensity, damage, or risk and includes both objective event factors and the subjective experience of the person.</t>
+        </is>
+      </c>
       <c r="F28" s="2" t="n"/>
       <c r="G28" s="2" t="n"/>
       <c r="H28" s="2" t="n"/>
-      <c r="I28" s="2" t="n"/>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>intensity</t>
+        </is>
+      </c>
       <c r="J28" s="2" t="n"/>
       <c r="K28" s="2" t="n"/>
       <c r="L28" s="2" t="inlineStr">
@@ -1754,7 +1746,7 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>include sub-classes for chronicity, frequency, duration, age at onset</t>
+          <t>Severity might be seen as a combination of several other attributes listed here - but I think we often think of this as an independent dimension.  Should there be sub-classes for obective severity and subjective or perceived severity, or for objective and perceived life threat?   - to be discussed with colleagues</t>
         </is>
       </c>
       <c r="O28" s="2" t="n"/>
@@ -1768,100 +1760,126 @@
       <c r="S28" s="2" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>TSTO:0000019</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>potentially traumatic experience time course</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>A &lt;potentially traumatic experience attribute&gt; that is the chronicity, duration, and frequency of the event(s) experienced.</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>potentially traumatic experience attribute</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="n"/>
+      <c r="H29" s="2" t="n"/>
+      <c r="I29" s="2" t="n"/>
+      <c r="J29" s="2" t="n"/>
+      <c r="K29" s="2" t="n"/>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>Pre-proposed</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>dimension</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>include sub-classes for chronicity, frequency, duration, age at onset</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="n"/>
+      <c r="P29" s="2" t="n"/>
+      <c r="Q29" s="2" t="inlineStr">
+        <is>
+          <t>NKA</t>
+        </is>
+      </c>
+      <c r="R29" s="2" t="n"/>
+      <c r="S29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>TSTO:0000020</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>potentially traumatic experience type</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>An attribute of a potentially traumatic experience that is the type of event(s) experienced by a person.</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>potentially traumatic experience attribute</t>
         </is>
       </c>
-      <c r="E29" s="4" t="n"/>
-      <c r="F29" s="4" t="n"/>
-      <c r="G29" s="4" t="n"/>
-      <c r="H29" s="4" t="n"/>
-      <c r="I29" s="4" t="inlineStr">
+      <c r="E30" s="4" t="n"/>
+      <c r="F30" s="4" t="n"/>
+      <c r="G30" s="4" t="n"/>
+      <c r="H30" s="4" t="n"/>
+      <c r="I30" s="4" t="inlineStr">
         <is>
           <t>event type</t>
         </is>
       </c>
-      <c r="J29" s="4" t="n"/>
-      <c r="K29" s="4" t="n"/>
-      <c r="L29" s="4" t="inlineStr">
+      <c r="J30" s="4" t="n"/>
+      <c r="K30" s="4" t="n"/>
+      <c r="L30" s="4" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="M29" s="4" t="n"/>
-      <c r="N29" s="4" t="n"/>
-      <c r="O29" s="4" t="n"/>
-      <c r="P29" s="4" t="n"/>
-      <c r="Q29" s="4" t="inlineStr">
+      <c r="M30" s="4" t="n"/>
+      <c r="N30" s="4" t="n"/>
+      <c r="O30" s="4" t="n"/>
+      <c r="P30" s="4" t="n"/>
+      <c r="Q30" s="4" t="inlineStr">
         <is>
           <t>NKA; RW</t>
         </is>
       </c>
-      <c r="R29" s="4" t="n"/>
-      <c r="S29" s="4" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>BFO:0000015</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>process</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>An occurrent that has temporal proper parts and for some time t.</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>occurrent</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
+      <c r="R30" s="4" t="n"/>
+      <c r="S30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>BCIO:043000</t>
+          <t>BFO:0000015</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>process attribute</t>
+          <t>process</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>A process profile that is an attribute of a process.</t>
+          <t>An occurrent that has temporal proper parts and for some time t.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>process profile</t>
+          <t>occurrent</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -1873,70 +1891,97 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>BCIO:043000</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>process attribute</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>A process profile that is an attribute of a process.</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>process profile</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>BFO:0000144</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>process profile</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>b is a process_profile =Def. there is some process c such that b process_profile_of c (axiom label in BFO2 Reference: [093-002])</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="2" t="n"/>
-      <c r="B33" s="2" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="2" t="n"/>
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>subjective severity of potentially traumatic experience</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>&lt;Potentially traumatic experience severity&gt; that is subjectively experienced by a person.</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>potentially traumatic experience severity</t>
         </is>
       </c>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="2" t="n"/>
-      <c r="G33" s="2" t="n"/>
-      <c r="H33" s="2" t="n"/>
-      <c r="I33" s="2" t="n"/>
-      <c r="J33" s="2" t="n"/>
-      <c r="K33" s="2" t="n"/>
-      <c r="L33" s="2" t="inlineStr">
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="n"/>
+      <c r="I34" s="2" t="n"/>
+      <c r="J34" s="2" t="n"/>
+      <c r="K34" s="2" t="n"/>
+      <c r="L34" s="2" t="inlineStr">
         <is>
           <t>Pre-proposed</t>
         </is>
       </c>
-      <c r="M33" s="2" t="inlineStr">
+      <c r="M34" s="2" t="inlineStr">
         <is>
           <t>dimension</t>
         </is>
       </c>
-      <c r="N33" s="2" t="n"/>
-      <c r="O33" s="2" t="n"/>
-      <c r="P33" s="2" t="n"/>
-      <c r="Q33" s="2" t="n"/>
-      <c r="R33" s="2" t="n"/>
-      <c r="S33" s="2" t="n"/>
+      <c r="N34" s="2" t="n"/>
+      <c r="O34" s="2" t="n"/>
+      <c r="P34" s="2" t="n"/>
+      <c r="Q34" s="2" t="n"/>
+      <c r="R34" s="2" t="n"/>
+      <c r="S34" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>